<commit_message>
Fix in pie-chart and pdf format
</commit_message>
<xml_diff>
--- a/backend/cerc_downloads/2025-09/MMC_Report_2025-09.xlsx
+++ b/backend/cerc_downloads/2025-09/MMC_Report_2025-09.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahesh Khicher\CERC Work\Market Monitoring Reports\Monthly\Sept 2025\For Publication-Revised\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05C341E-DFAA-44E0-86D5-EB3ADDBD97CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="849" firstSheet="13" activeTab="25"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11535" tabRatio="849" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table-1" sheetId="7" r:id="rId1"/>
@@ -3672,7 +3678,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="14">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
@@ -5329,11 +5335,47 @@
     <xf numFmtId="0" fontId="49" fillId="3" borderId="2" xfId="57" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="51" fillId="6" borderId="3" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="6" borderId="4" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="6" borderId="5" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="6" borderId="2" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="13" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="3" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="21" fillId="3" borderId="3" xfId="40" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="21" fillId="3" borderId="5" xfId="40" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -5345,46 +5387,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="6" borderId="3" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="3" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="8" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="6" borderId="3" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="6" borderId="4" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="6" borderId="4" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="6" borderId="5" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="13" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="6" borderId="2" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="6" borderId="3" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5518,6 +5524,9 @@
     <xf numFmtId="0" fontId="33" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5525,6 +5534,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5536,17 +5548,8 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="50" fillId="6" borderId="5" xfId="39" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5593,17 +5596,38 @@
     <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="50" fillId="6" borderId="2" xfId="39" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="50" fillId="6" borderId="2" xfId="39" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="28" fillId="4" borderId="2" xfId="39" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5623,6 +5647,12 @@
     <xf numFmtId="167" fontId="28" fillId="4" borderId="5" xfId="39" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5632,339 +5662,315 @@
     <xf numFmtId="0" fontId="28" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="307">
     <cellStyle name="Comma" xfId="61" builtinId="3"/>
-    <cellStyle name="Comma 12" xfId="62"/>
-    <cellStyle name="Comma 2" xfId="1"/>
-    <cellStyle name="Comma 2 10" xfId="63"/>
-    <cellStyle name="Comma 2 11" xfId="64"/>
-    <cellStyle name="Comma 2 12" xfId="65"/>
-    <cellStyle name="Comma 2 13" xfId="66"/>
-    <cellStyle name="Comma 2 14" xfId="67"/>
-    <cellStyle name="Comma 2 15" xfId="68"/>
-    <cellStyle name="Comma 2 16" xfId="69"/>
-    <cellStyle name="Comma 2 17" xfId="70"/>
-    <cellStyle name="Comma 2 18" xfId="71"/>
-    <cellStyle name="Comma 2 19" xfId="72"/>
-    <cellStyle name="Comma 2 2" xfId="73"/>
-    <cellStyle name="Comma 2 2 10" xfId="74"/>
-    <cellStyle name="Comma 2 2 2" xfId="75"/>
-    <cellStyle name="Comma 2 2 3" xfId="76"/>
-    <cellStyle name="Comma 2 2 4" xfId="77"/>
-    <cellStyle name="Comma 2 2 5" xfId="78"/>
-    <cellStyle name="Comma 2 2 6" xfId="79"/>
-    <cellStyle name="Comma 2 2 7" xfId="80"/>
-    <cellStyle name="Comma 2 2 8" xfId="81"/>
-    <cellStyle name="Comma 2 2 9" xfId="82"/>
-    <cellStyle name="Comma 2 20" xfId="83"/>
-    <cellStyle name="Comma 2 21" xfId="84"/>
-    <cellStyle name="Comma 2 22" xfId="85"/>
-    <cellStyle name="Comma 2 23" xfId="279"/>
-    <cellStyle name="Comma 2 3" xfId="86"/>
-    <cellStyle name="Comma 2 4" xfId="87"/>
-    <cellStyle name="Comma 2 5" xfId="88"/>
-    <cellStyle name="Comma 2 6" xfId="89"/>
-    <cellStyle name="Comma 2 7" xfId="90"/>
-    <cellStyle name="Comma 2 8" xfId="91"/>
-    <cellStyle name="Comma 2 9" xfId="92"/>
-    <cellStyle name="Comma 3" xfId="58"/>
-    <cellStyle name="Comma 3 10" xfId="93"/>
-    <cellStyle name="Comma 3 11" xfId="278"/>
-    <cellStyle name="Comma 3 2" xfId="94"/>
-    <cellStyle name="Comma 3 3" xfId="95"/>
-    <cellStyle name="Comma 3 4" xfId="96"/>
-    <cellStyle name="Comma 3 5" xfId="97"/>
-    <cellStyle name="Comma 3 6" xfId="98"/>
-    <cellStyle name="Comma 3 7" xfId="99"/>
-    <cellStyle name="Comma 3 8" xfId="100"/>
-    <cellStyle name="Comma 3 9" xfId="101"/>
-    <cellStyle name="Currency 2" xfId="2"/>
-    <cellStyle name="Currency 3" xfId="3"/>
-    <cellStyle name="Currency 3 2" xfId="4"/>
-    <cellStyle name="Currency 3 3" xfId="5"/>
-    <cellStyle name="Good 2" xfId="6"/>
-    <cellStyle name="Good 2 2" xfId="274"/>
-    <cellStyle name="Heading 2 2" xfId="7"/>
-    <cellStyle name="Heading 4 2" xfId="8"/>
+    <cellStyle name="Comma 12" xfId="62" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Comma 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Comma 2 10" xfId="63" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Comma 2 11" xfId="64" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Comma 2 12" xfId="65" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Comma 2 13" xfId="66" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Comma 2 14" xfId="67" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Comma 2 15" xfId="68" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Comma 2 16" xfId="69" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Comma 2 17" xfId="70" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Comma 2 18" xfId="71" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Comma 2 19" xfId="72" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Comma 2 2" xfId="73" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Comma 2 2 10" xfId="74" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Comma 2 2 2" xfId="75" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Comma 2 2 3" xfId="76" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Comma 2 2 4" xfId="77" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Comma 2 2 5" xfId="78" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="Comma 2 2 6" xfId="79" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="Comma 2 2 7" xfId="80" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="Comma 2 2 8" xfId="81" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="Comma 2 2 9" xfId="82" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Comma 2 20" xfId="83" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="Comma 2 21" xfId="84" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Comma 2 22" xfId="85" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Comma 2 23" xfId="279" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="Comma 2 3" xfId="86" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="Comma 2 4" xfId="87" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="Comma 2 5" xfId="88" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Comma 2 6" xfId="89" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="Comma 2 7" xfId="90" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="Comma 2 8" xfId="91" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="Comma 2 9" xfId="92" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="Comma 3" xfId="58" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Comma 3 10" xfId="93" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="Comma 3 11" xfId="278" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="Comma 3 2" xfId="94" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Comma 3 3" xfId="95" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="Comma 3 4" xfId="96" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
+    <cellStyle name="Comma 3 5" xfId="97" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
+    <cellStyle name="Comma 3 6" xfId="98" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
+    <cellStyle name="Comma 3 7" xfId="99" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
+    <cellStyle name="Comma 3 8" xfId="100" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
+    <cellStyle name="Comma 3 9" xfId="101" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
+    <cellStyle name="Currency 2" xfId="2" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
+    <cellStyle name="Currency 3" xfId="3" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
+    <cellStyle name="Currency 3 2" xfId="4" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
+    <cellStyle name="Currency 3 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
+    <cellStyle name="Good 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="Good 2 2" xfId="274" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
+    <cellStyle name="Heading 2 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
+    <cellStyle name="Heading 4 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="9"/>
-    <cellStyle name="Normal 10 2" xfId="301"/>
-    <cellStyle name="Normal 10 5" xfId="303"/>
-    <cellStyle name="Normal 11" xfId="59"/>
-    <cellStyle name="Normal 11 2" xfId="102"/>
-    <cellStyle name="Normal 12" xfId="103"/>
-    <cellStyle name="Normal 13" xfId="10"/>
-    <cellStyle name="Normal 13 2" xfId="294"/>
-    <cellStyle name="Normal 14" xfId="11"/>
-    <cellStyle name="Normal 14 10" xfId="104"/>
-    <cellStyle name="Normal 14 2" xfId="105"/>
-    <cellStyle name="Normal 14 3" xfId="106"/>
-    <cellStyle name="Normal 14 4" xfId="107"/>
-    <cellStyle name="Normal 14 5" xfId="108"/>
-    <cellStyle name="Normal 14 6" xfId="109"/>
-    <cellStyle name="Normal 14 7" xfId="110"/>
-    <cellStyle name="Normal 14 8" xfId="111"/>
-    <cellStyle name="Normal 14 9" xfId="112"/>
-    <cellStyle name="Normal 15" xfId="12"/>
-    <cellStyle name="Normal 15 2" xfId="289"/>
-    <cellStyle name="Normal 16" xfId="13"/>
-    <cellStyle name="Normal 17" xfId="113"/>
-    <cellStyle name="Normal 17 4" xfId="14"/>
-    <cellStyle name="Normal 18" xfId="270"/>
-    <cellStyle name="Normal 19" xfId="114"/>
-    <cellStyle name="Normal 2" xfId="15"/>
-    <cellStyle name="Normal 2 10" xfId="115"/>
-    <cellStyle name="Normal 2 11" xfId="116"/>
-    <cellStyle name="Normal 2 12" xfId="117"/>
-    <cellStyle name="Normal 2 13" xfId="118"/>
-    <cellStyle name="Normal 2 14" xfId="119"/>
-    <cellStyle name="Normal 2 15" xfId="120"/>
-    <cellStyle name="Normal 2 16" xfId="121"/>
-    <cellStyle name="Normal 2 17" xfId="122"/>
-    <cellStyle name="Normal 2 18" xfId="123"/>
-    <cellStyle name="Normal 2 19" xfId="124"/>
-    <cellStyle name="Normal 2 2" xfId="16"/>
-    <cellStyle name="Normal 2 2 10" xfId="125"/>
-    <cellStyle name="Normal 2 2 11" xfId="126"/>
-    <cellStyle name="Normal 2 2 12" xfId="127"/>
-    <cellStyle name="Normal 2 2 13" xfId="128"/>
-    <cellStyle name="Normal 2 2 14" xfId="129"/>
-    <cellStyle name="Normal 2 2 15" xfId="130"/>
-    <cellStyle name="Normal 2 2 16" xfId="131"/>
-    <cellStyle name="Normal 2 2 17" xfId="132"/>
-    <cellStyle name="Normal 2 2 18" xfId="273"/>
-    <cellStyle name="Normal 2 2 2" xfId="17"/>
-    <cellStyle name="Normal 2 2 2 10" xfId="133"/>
-    <cellStyle name="Normal 2 2 2 11" xfId="134"/>
-    <cellStyle name="Normal 2 2 2 12" xfId="135"/>
-    <cellStyle name="Normal 2 2 2 13" xfId="136"/>
-    <cellStyle name="Normal 2 2 2 14" xfId="275"/>
-    <cellStyle name="Normal 2 2 2 2" xfId="137"/>
-    <cellStyle name="Normal 2 2 2 2 3" xfId="291"/>
-    <cellStyle name="Normal 2 2 2 3" xfId="138"/>
-    <cellStyle name="Normal 2 2 2 4" xfId="139"/>
-    <cellStyle name="Normal 2 2 2 5" xfId="140"/>
-    <cellStyle name="Normal 2 2 2 6" xfId="141"/>
-    <cellStyle name="Normal 2 2 2 7" xfId="142"/>
-    <cellStyle name="Normal 2 2 2 8" xfId="143"/>
-    <cellStyle name="Normal 2 2 2 9" xfId="144"/>
-    <cellStyle name="Normal 2 2 3" xfId="18"/>
-    <cellStyle name="Normal 2 2 4" xfId="19"/>
-    <cellStyle name="Normal 2 2 5" xfId="20"/>
-    <cellStyle name="Normal 2 2 6" xfId="145"/>
-    <cellStyle name="Normal 2 2 7" xfId="146"/>
-    <cellStyle name="Normal 2 2 8" xfId="147"/>
-    <cellStyle name="Normal 2 2 9" xfId="148"/>
-    <cellStyle name="Normal 2 20" xfId="149"/>
-    <cellStyle name="Normal 2 21" xfId="150"/>
-    <cellStyle name="Normal 2 22" xfId="151"/>
-    <cellStyle name="Normal 2 23" xfId="152"/>
-    <cellStyle name="Normal 2 24" xfId="153"/>
-    <cellStyle name="Normal 2 25" xfId="154"/>
-    <cellStyle name="Normal 2 26" xfId="155"/>
-    <cellStyle name="Normal 2 27" xfId="156"/>
-    <cellStyle name="Normal 2 28" xfId="157"/>
-    <cellStyle name="Normal 2 29" xfId="158"/>
-    <cellStyle name="Normal 2 3" xfId="21"/>
-    <cellStyle name="Normal 2 3 10" xfId="159"/>
-    <cellStyle name="Normal 2 3 11" xfId="160"/>
-    <cellStyle name="Normal 2 3 2" xfId="60"/>
-    <cellStyle name="Normal 2 3 3" xfId="161"/>
-    <cellStyle name="Normal 2 3 4" xfId="162"/>
-    <cellStyle name="Normal 2 3 5" xfId="163"/>
-    <cellStyle name="Normal 2 3 6" xfId="164"/>
-    <cellStyle name="Normal 2 3 7" xfId="165"/>
-    <cellStyle name="Normal 2 3 8" xfId="166"/>
-    <cellStyle name="Normal 2 3 9" xfId="167"/>
-    <cellStyle name="Normal 2 30" xfId="168"/>
-    <cellStyle name="Normal 2 31" xfId="169"/>
-    <cellStyle name="Normal 2 32" xfId="170"/>
-    <cellStyle name="Normal 2 33" xfId="171"/>
-    <cellStyle name="Normal 2 34" xfId="172"/>
-    <cellStyle name="Normal 2 35" xfId="173"/>
-    <cellStyle name="Normal 2 36" xfId="174"/>
-    <cellStyle name="Normal 2 37" xfId="175"/>
-    <cellStyle name="Normal 2 38" xfId="176"/>
-    <cellStyle name="Normal 2 39" xfId="177"/>
-    <cellStyle name="Normal 2 4" xfId="22"/>
-    <cellStyle name="Normal 2 40" xfId="178"/>
-    <cellStyle name="Normal 2 41" xfId="179"/>
-    <cellStyle name="Normal 2 42" xfId="180"/>
-    <cellStyle name="Normal 2 43" xfId="181"/>
-    <cellStyle name="Normal 2 44" xfId="182"/>
-    <cellStyle name="Normal 2 45" xfId="183"/>
-    <cellStyle name="Normal 2 46" xfId="184"/>
-    <cellStyle name="Normal 2 47" xfId="185"/>
-    <cellStyle name="Normal 2 48" xfId="186"/>
-    <cellStyle name="Normal 2 49" xfId="187"/>
-    <cellStyle name="Normal 2 5" xfId="23"/>
-    <cellStyle name="Normal 2 50" xfId="188"/>
-    <cellStyle name="Normal 2 51" xfId="189"/>
-    <cellStyle name="Normal 2 52" xfId="190"/>
-    <cellStyle name="Normal 2 53" xfId="191"/>
-    <cellStyle name="Normal 2 54" xfId="272"/>
-    <cellStyle name="Normal 2 6" xfId="24"/>
-    <cellStyle name="Normal 2 7" xfId="192"/>
-    <cellStyle name="Normal 2 8" xfId="193"/>
-    <cellStyle name="Normal 2 9" xfId="194"/>
-    <cellStyle name="Normal 20" xfId="25"/>
-    <cellStyle name="Normal 21" xfId="26"/>
-    <cellStyle name="Normal 23" xfId="195"/>
-    <cellStyle name="Normal 27" xfId="196"/>
-    <cellStyle name="Normal 28" xfId="197"/>
-    <cellStyle name="Normal 29" xfId="198"/>
-    <cellStyle name="Normal 3" xfId="27"/>
-    <cellStyle name="Normal 3 2" xfId="28"/>
-    <cellStyle name="Normal 3 2 10" xfId="199"/>
-    <cellStyle name="Normal 3 2 2" xfId="200"/>
-    <cellStyle name="Normal 3 2 2 2" xfId="280"/>
-    <cellStyle name="Normal 3 2 3" xfId="201"/>
-    <cellStyle name="Normal 3 2 4" xfId="202"/>
-    <cellStyle name="Normal 3 2 5" xfId="203"/>
-    <cellStyle name="Normal 3 2 6" xfId="204"/>
-    <cellStyle name="Normal 3 2 7" xfId="205"/>
-    <cellStyle name="Normal 3 2 8" xfId="206"/>
-    <cellStyle name="Normal 3 2 9" xfId="207"/>
-    <cellStyle name="Normal 3 3" xfId="29"/>
-    <cellStyle name="Normal 3 4" xfId="30"/>
-    <cellStyle name="Normal 3 5" xfId="31"/>
-    <cellStyle name="Normal 3 6" xfId="32"/>
-    <cellStyle name="Normal 3 7" xfId="208"/>
-    <cellStyle name="Normal 30" xfId="209"/>
-    <cellStyle name="Normal 31" xfId="210"/>
-    <cellStyle name="Normal 32" xfId="211"/>
-    <cellStyle name="Normal 33" xfId="212"/>
-    <cellStyle name="Normal 34" xfId="213"/>
-    <cellStyle name="Normal 35" xfId="214"/>
-    <cellStyle name="Normal 36" xfId="215"/>
-    <cellStyle name="Normal 37" xfId="216"/>
-    <cellStyle name="Normal 4" xfId="33"/>
-    <cellStyle name="Normal 4 10" xfId="217"/>
-    <cellStyle name="Normal 4 11" xfId="218"/>
-    <cellStyle name="Normal 4 12" xfId="219"/>
-    <cellStyle name="Normal 4 13" xfId="220"/>
-    <cellStyle name="Normal 4 14" xfId="221"/>
-    <cellStyle name="Normal 4 15" xfId="222"/>
-    <cellStyle name="Normal 4 2" xfId="34"/>
-    <cellStyle name="Normal 4 3" xfId="35"/>
-    <cellStyle name="Normal 4 4" xfId="36"/>
-    <cellStyle name="Normal 4 5" xfId="37"/>
-    <cellStyle name="Normal 4 6" xfId="223"/>
-    <cellStyle name="Normal 4 7" xfId="224"/>
-    <cellStyle name="Normal 4 8" xfId="225"/>
-    <cellStyle name="Normal 4 9" xfId="226"/>
-    <cellStyle name="Normal 40" xfId="295"/>
-    <cellStyle name="Normal 43" xfId="281"/>
-    <cellStyle name="Normal 45" xfId="296"/>
-    <cellStyle name="Normal 47" xfId="38"/>
-    <cellStyle name="Normal 5" xfId="39"/>
-    <cellStyle name="Normal 5 2" xfId="227"/>
-    <cellStyle name="Normal 5 3" xfId="276"/>
-    <cellStyle name="Normal 50" xfId="282"/>
-    <cellStyle name="Normal 51" xfId="298"/>
-    <cellStyle name="Normal 55" xfId="297"/>
-    <cellStyle name="Normal 57" xfId="283"/>
-    <cellStyle name="Normal 59" xfId="299"/>
-    <cellStyle name="Normal 6" xfId="40"/>
-    <cellStyle name="Normal 63" xfId="41"/>
-    <cellStyle name="Normal 68" xfId="292"/>
-    <cellStyle name="Normal 69" xfId="286"/>
-    <cellStyle name="Normal 7" xfId="42"/>
-    <cellStyle name="Normal 7 10" xfId="228"/>
-    <cellStyle name="Normal 7 2" xfId="229"/>
-    <cellStyle name="Normal 7 3" xfId="230"/>
-    <cellStyle name="Normal 7 4" xfId="231"/>
-    <cellStyle name="Normal 7 5" xfId="232"/>
-    <cellStyle name="Normal 7 6" xfId="233"/>
-    <cellStyle name="Normal 7 7" xfId="234"/>
-    <cellStyle name="Normal 7 8" xfId="235"/>
-    <cellStyle name="Normal 7 9" xfId="236"/>
-    <cellStyle name="Normal 70" xfId="290"/>
-    <cellStyle name="Normal 72" xfId="288"/>
-    <cellStyle name="Normal 73" xfId="287"/>
-    <cellStyle name="Normal 74" xfId="285"/>
-    <cellStyle name="Normal 75" xfId="284"/>
-    <cellStyle name="Normal 78" xfId="293"/>
-    <cellStyle name="Normal 8" xfId="43"/>
-    <cellStyle name="Normal 8 2" xfId="271"/>
-    <cellStyle name="Normal 88" xfId="300"/>
-    <cellStyle name="Normal 9" xfId="44"/>
-    <cellStyle name="Normal 90" xfId="302"/>
-    <cellStyle name="Normal 91" xfId="304"/>
-    <cellStyle name="Normal 92" xfId="305"/>
-    <cellStyle name="Normal 94" xfId="306"/>
-    <cellStyle name="Normal_MMC Monthly Report Apr 2010 2" xfId="57"/>
+    <cellStyle name="Normal 10" xfId="9" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
+    <cellStyle name="Normal 10 2" xfId="301" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
+    <cellStyle name="Normal 10 5" xfId="303" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
+    <cellStyle name="Normal 11" xfId="59" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
+    <cellStyle name="Normal 11 2" xfId="102" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
+    <cellStyle name="Normal 12" xfId="103" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
+    <cellStyle name="Normal 13" xfId="10" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
+    <cellStyle name="Normal 13 2" xfId="294" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
+    <cellStyle name="Normal 14" xfId="11" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
+    <cellStyle name="Normal 14 10" xfId="104" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
+    <cellStyle name="Normal 14 2" xfId="105" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
+    <cellStyle name="Normal 14 3" xfId="106" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
+    <cellStyle name="Normal 14 4" xfId="107" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
+    <cellStyle name="Normal 14 5" xfId="108" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
+    <cellStyle name="Normal 14 6" xfId="109" xr:uid="{00000000-0005-0000-0000-000044000000}"/>
+    <cellStyle name="Normal 14 7" xfId="110" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
+    <cellStyle name="Normal 14 8" xfId="111" xr:uid="{00000000-0005-0000-0000-000046000000}"/>
+    <cellStyle name="Normal 14 9" xfId="112" xr:uid="{00000000-0005-0000-0000-000047000000}"/>
+    <cellStyle name="Normal 15" xfId="12" xr:uid="{00000000-0005-0000-0000-000048000000}"/>
+    <cellStyle name="Normal 15 2" xfId="289" xr:uid="{00000000-0005-0000-0000-000049000000}"/>
+    <cellStyle name="Normal 16" xfId="13" xr:uid="{00000000-0005-0000-0000-00004A000000}"/>
+    <cellStyle name="Normal 17" xfId="113" xr:uid="{00000000-0005-0000-0000-00004B000000}"/>
+    <cellStyle name="Normal 17 4" xfId="14" xr:uid="{00000000-0005-0000-0000-00004C000000}"/>
+    <cellStyle name="Normal 18" xfId="270" xr:uid="{00000000-0005-0000-0000-00004D000000}"/>
+    <cellStyle name="Normal 19" xfId="114" xr:uid="{00000000-0005-0000-0000-00004E000000}"/>
+    <cellStyle name="Normal 2" xfId="15" xr:uid="{00000000-0005-0000-0000-00004F000000}"/>
+    <cellStyle name="Normal 2 10" xfId="115" xr:uid="{00000000-0005-0000-0000-000050000000}"/>
+    <cellStyle name="Normal 2 11" xfId="116" xr:uid="{00000000-0005-0000-0000-000051000000}"/>
+    <cellStyle name="Normal 2 12" xfId="117" xr:uid="{00000000-0005-0000-0000-000052000000}"/>
+    <cellStyle name="Normal 2 13" xfId="118" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
+    <cellStyle name="Normal 2 14" xfId="119" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
+    <cellStyle name="Normal 2 15" xfId="120" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
+    <cellStyle name="Normal 2 16" xfId="121" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
+    <cellStyle name="Normal 2 17" xfId="122" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
+    <cellStyle name="Normal 2 18" xfId="123" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
+    <cellStyle name="Normal 2 19" xfId="124" xr:uid="{00000000-0005-0000-0000-000059000000}"/>
+    <cellStyle name="Normal 2 2" xfId="16" xr:uid="{00000000-0005-0000-0000-00005A000000}"/>
+    <cellStyle name="Normal 2 2 10" xfId="125" xr:uid="{00000000-0005-0000-0000-00005B000000}"/>
+    <cellStyle name="Normal 2 2 11" xfId="126" xr:uid="{00000000-0005-0000-0000-00005C000000}"/>
+    <cellStyle name="Normal 2 2 12" xfId="127" xr:uid="{00000000-0005-0000-0000-00005D000000}"/>
+    <cellStyle name="Normal 2 2 13" xfId="128" xr:uid="{00000000-0005-0000-0000-00005E000000}"/>
+    <cellStyle name="Normal 2 2 14" xfId="129" xr:uid="{00000000-0005-0000-0000-00005F000000}"/>
+    <cellStyle name="Normal 2 2 15" xfId="130" xr:uid="{00000000-0005-0000-0000-000060000000}"/>
+    <cellStyle name="Normal 2 2 16" xfId="131" xr:uid="{00000000-0005-0000-0000-000061000000}"/>
+    <cellStyle name="Normal 2 2 17" xfId="132" xr:uid="{00000000-0005-0000-0000-000062000000}"/>
+    <cellStyle name="Normal 2 2 18" xfId="273" xr:uid="{00000000-0005-0000-0000-000063000000}"/>
+    <cellStyle name="Normal 2 2 2" xfId="17" xr:uid="{00000000-0005-0000-0000-000064000000}"/>
+    <cellStyle name="Normal 2 2 2 10" xfId="133" xr:uid="{00000000-0005-0000-0000-000065000000}"/>
+    <cellStyle name="Normal 2 2 2 11" xfId="134" xr:uid="{00000000-0005-0000-0000-000066000000}"/>
+    <cellStyle name="Normal 2 2 2 12" xfId="135" xr:uid="{00000000-0005-0000-0000-000067000000}"/>
+    <cellStyle name="Normal 2 2 2 13" xfId="136" xr:uid="{00000000-0005-0000-0000-000068000000}"/>
+    <cellStyle name="Normal 2 2 2 14" xfId="275" xr:uid="{00000000-0005-0000-0000-000069000000}"/>
+    <cellStyle name="Normal 2 2 2 2" xfId="137" xr:uid="{00000000-0005-0000-0000-00006A000000}"/>
+    <cellStyle name="Normal 2 2 2 2 3" xfId="291" xr:uid="{00000000-0005-0000-0000-00006B000000}"/>
+    <cellStyle name="Normal 2 2 2 3" xfId="138" xr:uid="{00000000-0005-0000-0000-00006C000000}"/>
+    <cellStyle name="Normal 2 2 2 4" xfId="139" xr:uid="{00000000-0005-0000-0000-00006D000000}"/>
+    <cellStyle name="Normal 2 2 2 5" xfId="140" xr:uid="{00000000-0005-0000-0000-00006E000000}"/>
+    <cellStyle name="Normal 2 2 2 6" xfId="141" xr:uid="{00000000-0005-0000-0000-00006F000000}"/>
+    <cellStyle name="Normal 2 2 2 7" xfId="142" xr:uid="{00000000-0005-0000-0000-000070000000}"/>
+    <cellStyle name="Normal 2 2 2 8" xfId="143" xr:uid="{00000000-0005-0000-0000-000071000000}"/>
+    <cellStyle name="Normal 2 2 2 9" xfId="144" xr:uid="{00000000-0005-0000-0000-000072000000}"/>
+    <cellStyle name="Normal 2 2 3" xfId="18" xr:uid="{00000000-0005-0000-0000-000073000000}"/>
+    <cellStyle name="Normal 2 2 4" xfId="19" xr:uid="{00000000-0005-0000-0000-000074000000}"/>
+    <cellStyle name="Normal 2 2 5" xfId="20" xr:uid="{00000000-0005-0000-0000-000075000000}"/>
+    <cellStyle name="Normal 2 2 6" xfId="145" xr:uid="{00000000-0005-0000-0000-000076000000}"/>
+    <cellStyle name="Normal 2 2 7" xfId="146" xr:uid="{00000000-0005-0000-0000-000077000000}"/>
+    <cellStyle name="Normal 2 2 8" xfId="147" xr:uid="{00000000-0005-0000-0000-000078000000}"/>
+    <cellStyle name="Normal 2 2 9" xfId="148" xr:uid="{00000000-0005-0000-0000-000079000000}"/>
+    <cellStyle name="Normal 2 20" xfId="149" xr:uid="{00000000-0005-0000-0000-00007A000000}"/>
+    <cellStyle name="Normal 2 21" xfId="150" xr:uid="{00000000-0005-0000-0000-00007B000000}"/>
+    <cellStyle name="Normal 2 22" xfId="151" xr:uid="{00000000-0005-0000-0000-00007C000000}"/>
+    <cellStyle name="Normal 2 23" xfId="152" xr:uid="{00000000-0005-0000-0000-00007D000000}"/>
+    <cellStyle name="Normal 2 24" xfId="153" xr:uid="{00000000-0005-0000-0000-00007E000000}"/>
+    <cellStyle name="Normal 2 25" xfId="154" xr:uid="{00000000-0005-0000-0000-00007F000000}"/>
+    <cellStyle name="Normal 2 26" xfId="155" xr:uid="{00000000-0005-0000-0000-000080000000}"/>
+    <cellStyle name="Normal 2 27" xfId="156" xr:uid="{00000000-0005-0000-0000-000081000000}"/>
+    <cellStyle name="Normal 2 28" xfId="157" xr:uid="{00000000-0005-0000-0000-000082000000}"/>
+    <cellStyle name="Normal 2 29" xfId="158" xr:uid="{00000000-0005-0000-0000-000083000000}"/>
+    <cellStyle name="Normal 2 3" xfId="21" xr:uid="{00000000-0005-0000-0000-000084000000}"/>
+    <cellStyle name="Normal 2 3 10" xfId="159" xr:uid="{00000000-0005-0000-0000-000085000000}"/>
+    <cellStyle name="Normal 2 3 11" xfId="160" xr:uid="{00000000-0005-0000-0000-000086000000}"/>
+    <cellStyle name="Normal 2 3 2" xfId="60" xr:uid="{00000000-0005-0000-0000-000087000000}"/>
+    <cellStyle name="Normal 2 3 3" xfId="161" xr:uid="{00000000-0005-0000-0000-000088000000}"/>
+    <cellStyle name="Normal 2 3 4" xfId="162" xr:uid="{00000000-0005-0000-0000-000089000000}"/>
+    <cellStyle name="Normal 2 3 5" xfId="163" xr:uid="{00000000-0005-0000-0000-00008A000000}"/>
+    <cellStyle name="Normal 2 3 6" xfId="164" xr:uid="{00000000-0005-0000-0000-00008B000000}"/>
+    <cellStyle name="Normal 2 3 7" xfId="165" xr:uid="{00000000-0005-0000-0000-00008C000000}"/>
+    <cellStyle name="Normal 2 3 8" xfId="166" xr:uid="{00000000-0005-0000-0000-00008D000000}"/>
+    <cellStyle name="Normal 2 3 9" xfId="167" xr:uid="{00000000-0005-0000-0000-00008E000000}"/>
+    <cellStyle name="Normal 2 30" xfId="168" xr:uid="{00000000-0005-0000-0000-00008F000000}"/>
+    <cellStyle name="Normal 2 31" xfId="169" xr:uid="{00000000-0005-0000-0000-000090000000}"/>
+    <cellStyle name="Normal 2 32" xfId="170" xr:uid="{00000000-0005-0000-0000-000091000000}"/>
+    <cellStyle name="Normal 2 33" xfId="171" xr:uid="{00000000-0005-0000-0000-000092000000}"/>
+    <cellStyle name="Normal 2 34" xfId="172" xr:uid="{00000000-0005-0000-0000-000093000000}"/>
+    <cellStyle name="Normal 2 35" xfId="173" xr:uid="{00000000-0005-0000-0000-000094000000}"/>
+    <cellStyle name="Normal 2 36" xfId="174" xr:uid="{00000000-0005-0000-0000-000095000000}"/>
+    <cellStyle name="Normal 2 37" xfId="175" xr:uid="{00000000-0005-0000-0000-000096000000}"/>
+    <cellStyle name="Normal 2 38" xfId="176" xr:uid="{00000000-0005-0000-0000-000097000000}"/>
+    <cellStyle name="Normal 2 39" xfId="177" xr:uid="{00000000-0005-0000-0000-000098000000}"/>
+    <cellStyle name="Normal 2 4" xfId="22" xr:uid="{00000000-0005-0000-0000-000099000000}"/>
+    <cellStyle name="Normal 2 40" xfId="178" xr:uid="{00000000-0005-0000-0000-00009A000000}"/>
+    <cellStyle name="Normal 2 41" xfId="179" xr:uid="{00000000-0005-0000-0000-00009B000000}"/>
+    <cellStyle name="Normal 2 42" xfId="180" xr:uid="{00000000-0005-0000-0000-00009C000000}"/>
+    <cellStyle name="Normal 2 43" xfId="181" xr:uid="{00000000-0005-0000-0000-00009D000000}"/>
+    <cellStyle name="Normal 2 44" xfId="182" xr:uid="{00000000-0005-0000-0000-00009E000000}"/>
+    <cellStyle name="Normal 2 45" xfId="183" xr:uid="{00000000-0005-0000-0000-00009F000000}"/>
+    <cellStyle name="Normal 2 46" xfId="184" xr:uid="{00000000-0005-0000-0000-0000A0000000}"/>
+    <cellStyle name="Normal 2 47" xfId="185" xr:uid="{00000000-0005-0000-0000-0000A1000000}"/>
+    <cellStyle name="Normal 2 48" xfId="186" xr:uid="{00000000-0005-0000-0000-0000A2000000}"/>
+    <cellStyle name="Normal 2 49" xfId="187" xr:uid="{00000000-0005-0000-0000-0000A3000000}"/>
+    <cellStyle name="Normal 2 5" xfId="23" xr:uid="{00000000-0005-0000-0000-0000A4000000}"/>
+    <cellStyle name="Normal 2 50" xfId="188" xr:uid="{00000000-0005-0000-0000-0000A5000000}"/>
+    <cellStyle name="Normal 2 51" xfId="189" xr:uid="{00000000-0005-0000-0000-0000A6000000}"/>
+    <cellStyle name="Normal 2 52" xfId="190" xr:uid="{00000000-0005-0000-0000-0000A7000000}"/>
+    <cellStyle name="Normal 2 53" xfId="191" xr:uid="{00000000-0005-0000-0000-0000A8000000}"/>
+    <cellStyle name="Normal 2 54" xfId="272" xr:uid="{00000000-0005-0000-0000-0000A9000000}"/>
+    <cellStyle name="Normal 2 6" xfId="24" xr:uid="{00000000-0005-0000-0000-0000AA000000}"/>
+    <cellStyle name="Normal 2 7" xfId="192" xr:uid="{00000000-0005-0000-0000-0000AB000000}"/>
+    <cellStyle name="Normal 2 8" xfId="193" xr:uid="{00000000-0005-0000-0000-0000AC000000}"/>
+    <cellStyle name="Normal 2 9" xfId="194" xr:uid="{00000000-0005-0000-0000-0000AD000000}"/>
+    <cellStyle name="Normal 20" xfId="25" xr:uid="{00000000-0005-0000-0000-0000AE000000}"/>
+    <cellStyle name="Normal 21" xfId="26" xr:uid="{00000000-0005-0000-0000-0000AF000000}"/>
+    <cellStyle name="Normal 23" xfId="195" xr:uid="{00000000-0005-0000-0000-0000B0000000}"/>
+    <cellStyle name="Normal 27" xfId="196" xr:uid="{00000000-0005-0000-0000-0000B1000000}"/>
+    <cellStyle name="Normal 28" xfId="197" xr:uid="{00000000-0005-0000-0000-0000B2000000}"/>
+    <cellStyle name="Normal 29" xfId="198" xr:uid="{00000000-0005-0000-0000-0000B3000000}"/>
+    <cellStyle name="Normal 3" xfId="27" xr:uid="{00000000-0005-0000-0000-0000B4000000}"/>
+    <cellStyle name="Normal 3 2" xfId="28" xr:uid="{00000000-0005-0000-0000-0000B5000000}"/>
+    <cellStyle name="Normal 3 2 10" xfId="199" xr:uid="{00000000-0005-0000-0000-0000B6000000}"/>
+    <cellStyle name="Normal 3 2 2" xfId="200" xr:uid="{00000000-0005-0000-0000-0000B7000000}"/>
+    <cellStyle name="Normal 3 2 2 2" xfId="280" xr:uid="{00000000-0005-0000-0000-0000B8000000}"/>
+    <cellStyle name="Normal 3 2 3" xfId="201" xr:uid="{00000000-0005-0000-0000-0000B9000000}"/>
+    <cellStyle name="Normal 3 2 4" xfId="202" xr:uid="{00000000-0005-0000-0000-0000BA000000}"/>
+    <cellStyle name="Normal 3 2 5" xfId="203" xr:uid="{00000000-0005-0000-0000-0000BB000000}"/>
+    <cellStyle name="Normal 3 2 6" xfId="204" xr:uid="{00000000-0005-0000-0000-0000BC000000}"/>
+    <cellStyle name="Normal 3 2 7" xfId="205" xr:uid="{00000000-0005-0000-0000-0000BD000000}"/>
+    <cellStyle name="Normal 3 2 8" xfId="206" xr:uid="{00000000-0005-0000-0000-0000BE000000}"/>
+    <cellStyle name="Normal 3 2 9" xfId="207" xr:uid="{00000000-0005-0000-0000-0000BF000000}"/>
+    <cellStyle name="Normal 3 3" xfId="29" xr:uid="{00000000-0005-0000-0000-0000C0000000}"/>
+    <cellStyle name="Normal 3 4" xfId="30" xr:uid="{00000000-0005-0000-0000-0000C1000000}"/>
+    <cellStyle name="Normal 3 5" xfId="31" xr:uid="{00000000-0005-0000-0000-0000C2000000}"/>
+    <cellStyle name="Normal 3 6" xfId="32" xr:uid="{00000000-0005-0000-0000-0000C3000000}"/>
+    <cellStyle name="Normal 3 7" xfId="208" xr:uid="{00000000-0005-0000-0000-0000C4000000}"/>
+    <cellStyle name="Normal 30" xfId="209" xr:uid="{00000000-0005-0000-0000-0000C5000000}"/>
+    <cellStyle name="Normal 31" xfId="210" xr:uid="{00000000-0005-0000-0000-0000C6000000}"/>
+    <cellStyle name="Normal 32" xfId="211" xr:uid="{00000000-0005-0000-0000-0000C7000000}"/>
+    <cellStyle name="Normal 33" xfId="212" xr:uid="{00000000-0005-0000-0000-0000C8000000}"/>
+    <cellStyle name="Normal 34" xfId="213" xr:uid="{00000000-0005-0000-0000-0000C9000000}"/>
+    <cellStyle name="Normal 35" xfId="214" xr:uid="{00000000-0005-0000-0000-0000CA000000}"/>
+    <cellStyle name="Normal 36" xfId="215" xr:uid="{00000000-0005-0000-0000-0000CB000000}"/>
+    <cellStyle name="Normal 37" xfId="216" xr:uid="{00000000-0005-0000-0000-0000CC000000}"/>
+    <cellStyle name="Normal 4" xfId="33" xr:uid="{00000000-0005-0000-0000-0000CD000000}"/>
+    <cellStyle name="Normal 4 10" xfId="217" xr:uid="{00000000-0005-0000-0000-0000CE000000}"/>
+    <cellStyle name="Normal 4 11" xfId="218" xr:uid="{00000000-0005-0000-0000-0000CF000000}"/>
+    <cellStyle name="Normal 4 12" xfId="219" xr:uid="{00000000-0005-0000-0000-0000D0000000}"/>
+    <cellStyle name="Normal 4 13" xfId="220" xr:uid="{00000000-0005-0000-0000-0000D1000000}"/>
+    <cellStyle name="Normal 4 14" xfId="221" xr:uid="{00000000-0005-0000-0000-0000D2000000}"/>
+    <cellStyle name="Normal 4 15" xfId="222" xr:uid="{00000000-0005-0000-0000-0000D3000000}"/>
+    <cellStyle name="Normal 4 2" xfId="34" xr:uid="{00000000-0005-0000-0000-0000D4000000}"/>
+    <cellStyle name="Normal 4 3" xfId="35" xr:uid="{00000000-0005-0000-0000-0000D5000000}"/>
+    <cellStyle name="Normal 4 4" xfId="36" xr:uid="{00000000-0005-0000-0000-0000D6000000}"/>
+    <cellStyle name="Normal 4 5" xfId="37" xr:uid="{00000000-0005-0000-0000-0000D7000000}"/>
+    <cellStyle name="Normal 4 6" xfId="223" xr:uid="{00000000-0005-0000-0000-0000D8000000}"/>
+    <cellStyle name="Normal 4 7" xfId="224" xr:uid="{00000000-0005-0000-0000-0000D9000000}"/>
+    <cellStyle name="Normal 4 8" xfId="225" xr:uid="{00000000-0005-0000-0000-0000DA000000}"/>
+    <cellStyle name="Normal 4 9" xfId="226" xr:uid="{00000000-0005-0000-0000-0000DB000000}"/>
+    <cellStyle name="Normal 40" xfId="295" xr:uid="{00000000-0005-0000-0000-0000DC000000}"/>
+    <cellStyle name="Normal 43" xfId="281" xr:uid="{00000000-0005-0000-0000-0000DD000000}"/>
+    <cellStyle name="Normal 45" xfId="296" xr:uid="{00000000-0005-0000-0000-0000DE000000}"/>
+    <cellStyle name="Normal 47" xfId="38" xr:uid="{00000000-0005-0000-0000-0000DF000000}"/>
+    <cellStyle name="Normal 5" xfId="39" xr:uid="{00000000-0005-0000-0000-0000E0000000}"/>
+    <cellStyle name="Normal 5 2" xfId="227" xr:uid="{00000000-0005-0000-0000-0000E1000000}"/>
+    <cellStyle name="Normal 5 3" xfId="276" xr:uid="{00000000-0005-0000-0000-0000E2000000}"/>
+    <cellStyle name="Normal 50" xfId="282" xr:uid="{00000000-0005-0000-0000-0000E3000000}"/>
+    <cellStyle name="Normal 51" xfId="298" xr:uid="{00000000-0005-0000-0000-0000E4000000}"/>
+    <cellStyle name="Normal 55" xfId="297" xr:uid="{00000000-0005-0000-0000-0000E5000000}"/>
+    <cellStyle name="Normal 57" xfId="283" xr:uid="{00000000-0005-0000-0000-0000E6000000}"/>
+    <cellStyle name="Normal 59" xfId="299" xr:uid="{00000000-0005-0000-0000-0000E7000000}"/>
+    <cellStyle name="Normal 6" xfId="40" xr:uid="{00000000-0005-0000-0000-0000E8000000}"/>
+    <cellStyle name="Normal 63" xfId="41" xr:uid="{00000000-0005-0000-0000-0000E9000000}"/>
+    <cellStyle name="Normal 68" xfId="292" xr:uid="{00000000-0005-0000-0000-0000EA000000}"/>
+    <cellStyle name="Normal 69" xfId="286" xr:uid="{00000000-0005-0000-0000-0000EB000000}"/>
+    <cellStyle name="Normal 7" xfId="42" xr:uid="{00000000-0005-0000-0000-0000EC000000}"/>
+    <cellStyle name="Normal 7 10" xfId="228" xr:uid="{00000000-0005-0000-0000-0000ED000000}"/>
+    <cellStyle name="Normal 7 2" xfId="229" xr:uid="{00000000-0005-0000-0000-0000EE000000}"/>
+    <cellStyle name="Normal 7 3" xfId="230" xr:uid="{00000000-0005-0000-0000-0000EF000000}"/>
+    <cellStyle name="Normal 7 4" xfId="231" xr:uid="{00000000-0005-0000-0000-0000F0000000}"/>
+    <cellStyle name="Normal 7 5" xfId="232" xr:uid="{00000000-0005-0000-0000-0000F1000000}"/>
+    <cellStyle name="Normal 7 6" xfId="233" xr:uid="{00000000-0005-0000-0000-0000F2000000}"/>
+    <cellStyle name="Normal 7 7" xfId="234" xr:uid="{00000000-0005-0000-0000-0000F3000000}"/>
+    <cellStyle name="Normal 7 8" xfId="235" xr:uid="{00000000-0005-0000-0000-0000F4000000}"/>
+    <cellStyle name="Normal 7 9" xfId="236" xr:uid="{00000000-0005-0000-0000-0000F5000000}"/>
+    <cellStyle name="Normal 70" xfId="290" xr:uid="{00000000-0005-0000-0000-0000F6000000}"/>
+    <cellStyle name="Normal 72" xfId="288" xr:uid="{00000000-0005-0000-0000-0000F7000000}"/>
+    <cellStyle name="Normal 73" xfId="287" xr:uid="{00000000-0005-0000-0000-0000F8000000}"/>
+    <cellStyle name="Normal 74" xfId="285" xr:uid="{00000000-0005-0000-0000-0000F9000000}"/>
+    <cellStyle name="Normal 75" xfId="284" xr:uid="{00000000-0005-0000-0000-0000FA000000}"/>
+    <cellStyle name="Normal 78" xfId="293" xr:uid="{00000000-0005-0000-0000-0000FB000000}"/>
+    <cellStyle name="Normal 8" xfId="43" xr:uid="{00000000-0005-0000-0000-0000FC000000}"/>
+    <cellStyle name="Normal 8 2" xfId="271" xr:uid="{00000000-0005-0000-0000-0000FD000000}"/>
+    <cellStyle name="Normal 88" xfId="300" xr:uid="{00000000-0005-0000-0000-0000FE000000}"/>
+    <cellStyle name="Normal 9" xfId="44" xr:uid="{00000000-0005-0000-0000-0000FF000000}"/>
+    <cellStyle name="Normal 90" xfId="302" xr:uid="{00000000-0005-0000-0000-000000010000}"/>
+    <cellStyle name="Normal 91" xfId="304" xr:uid="{00000000-0005-0000-0000-000001010000}"/>
+    <cellStyle name="Normal 92" xfId="305" xr:uid="{00000000-0005-0000-0000-000002010000}"/>
+    <cellStyle name="Normal 94" xfId="306" xr:uid="{00000000-0005-0000-0000-000003010000}"/>
+    <cellStyle name="Normal_MMC Monthly Report Apr 2010 2" xfId="57" xr:uid="{00000000-0005-0000-0000-000004010000}"/>
     <cellStyle name="Percent" xfId="56" builtinId="5"/>
-    <cellStyle name="Percent 2" xfId="45"/>
-    <cellStyle name="Percent 2 10" xfId="237"/>
-    <cellStyle name="Percent 2 11" xfId="238"/>
-    <cellStyle name="Percent 2 12" xfId="239"/>
-    <cellStyle name="Percent 2 13" xfId="240"/>
-    <cellStyle name="Percent 2 14" xfId="241"/>
-    <cellStyle name="Percent 2 15" xfId="242"/>
-    <cellStyle name="Percent 2 16" xfId="243"/>
-    <cellStyle name="Percent 2 17" xfId="244"/>
-    <cellStyle name="Percent 2 18" xfId="245"/>
-    <cellStyle name="Percent 2 19" xfId="246"/>
-    <cellStyle name="Percent 2 2" xfId="46"/>
-    <cellStyle name="Percent 2 2 10" xfId="247"/>
-    <cellStyle name="Percent 2 2 11" xfId="248"/>
-    <cellStyle name="Percent 2 2 12" xfId="249"/>
-    <cellStyle name="Percent 2 2 13" xfId="250"/>
-    <cellStyle name="Percent 2 2 14" xfId="277"/>
-    <cellStyle name="Percent 2 2 2" xfId="251"/>
-    <cellStyle name="Percent 2 2 3" xfId="252"/>
-    <cellStyle name="Percent 2 2 4" xfId="253"/>
-    <cellStyle name="Percent 2 2 5" xfId="254"/>
-    <cellStyle name="Percent 2 2 6" xfId="255"/>
-    <cellStyle name="Percent 2 2 7" xfId="256"/>
-    <cellStyle name="Percent 2 2 8" xfId="257"/>
-    <cellStyle name="Percent 2 2 9" xfId="258"/>
-    <cellStyle name="Percent 2 20" xfId="259"/>
-    <cellStyle name="Percent 2 21" xfId="260"/>
-    <cellStyle name="Percent 2 22" xfId="261"/>
-    <cellStyle name="Percent 2 23" xfId="262"/>
-    <cellStyle name="Percent 2 24" xfId="263"/>
-    <cellStyle name="Percent 2 25" xfId="264"/>
-    <cellStyle name="Percent 2 3" xfId="47"/>
-    <cellStyle name="Percent 2 4" xfId="48"/>
-    <cellStyle name="Percent 2 5" xfId="49"/>
-    <cellStyle name="Percent 2 6" xfId="265"/>
-    <cellStyle name="Percent 2 7" xfId="266"/>
-    <cellStyle name="Percent 2 8" xfId="267"/>
-    <cellStyle name="Percent 2 9" xfId="268"/>
-    <cellStyle name="Percent 3" xfId="50"/>
-    <cellStyle name="Percent 3 2" xfId="51"/>
-    <cellStyle name="Percent 3 3" xfId="52"/>
-    <cellStyle name="Percent 3 4" xfId="53"/>
-    <cellStyle name="Percent 3 5" xfId="54"/>
-    <cellStyle name="Percent 4" xfId="55"/>
-    <cellStyle name="TableStyleLight1" xfId="269"/>
+    <cellStyle name="Percent 2" xfId="45" xr:uid="{00000000-0005-0000-0000-000006010000}"/>
+    <cellStyle name="Percent 2 10" xfId="237" xr:uid="{00000000-0005-0000-0000-000007010000}"/>
+    <cellStyle name="Percent 2 11" xfId="238" xr:uid="{00000000-0005-0000-0000-000008010000}"/>
+    <cellStyle name="Percent 2 12" xfId="239" xr:uid="{00000000-0005-0000-0000-000009010000}"/>
+    <cellStyle name="Percent 2 13" xfId="240" xr:uid="{00000000-0005-0000-0000-00000A010000}"/>
+    <cellStyle name="Percent 2 14" xfId="241" xr:uid="{00000000-0005-0000-0000-00000B010000}"/>
+    <cellStyle name="Percent 2 15" xfId="242" xr:uid="{00000000-0005-0000-0000-00000C010000}"/>
+    <cellStyle name="Percent 2 16" xfId="243" xr:uid="{00000000-0005-0000-0000-00000D010000}"/>
+    <cellStyle name="Percent 2 17" xfId="244" xr:uid="{00000000-0005-0000-0000-00000E010000}"/>
+    <cellStyle name="Percent 2 18" xfId="245" xr:uid="{00000000-0005-0000-0000-00000F010000}"/>
+    <cellStyle name="Percent 2 19" xfId="246" xr:uid="{00000000-0005-0000-0000-000010010000}"/>
+    <cellStyle name="Percent 2 2" xfId="46" xr:uid="{00000000-0005-0000-0000-000011010000}"/>
+    <cellStyle name="Percent 2 2 10" xfId="247" xr:uid="{00000000-0005-0000-0000-000012010000}"/>
+    <cellStyle name="Percent 2 2 11" xfId="248" xr:uid="{00000000-0005-0000-0000-000013010000}"/>
+    <cellStyle name="Percent 2 2 12" xfId="249" xr:uid="{00000000-0005-0000-0000-000014010000}"/>
+    <cellStyle name="Percent 2 2 13" xfId="250" xr:uid="{00000000-0005-0000-0000-000015010000}"/>
+    <cellStyle name="Percent 2 2 14" xfId="277" xr:uid="{00000000-0005-0000-0000-000016010000}"/>
+    <cellStyle name="Percent 2 2 2" xfId="251" xr:uid="{00000000-0005-0000-0000-000017010000}"/>
+    <cellStyle name="Percent 2 2 3" xfId="252" xr:uid="{00000000-0005-0000-0000-000018010000}"/>
+    <cellStyle name="Percent 2 2 4" xfId="253" xr:uid="{00000000-0005-0000-0000-000019010000}"/>
+    <cellStyle name="Percent 2 2 5" xfId="254" xr:uid="{00000000-0005-0000-0000-00001A010000}"/>
+    <cellStyle name="Percent 2 2 6" xfId="255" xr:uid="{00000000-0005-0000-0000-00001B010000}"/>
+    <cellStyle name="Percent 2 2 7" xfId="256" xr:uid="{00000000-0005-0000-0000-00001C010000}"/>
+    <cellStyle name="Percent 2 2 8" xfId="257" xr:uid="{00000000-0005-0000-0000-00001D010000}"/>
+    <cellStyle name="Percent 2 2 9" xfId="258" xr:uid="{00000000-0005-0000-0000-00001E010000}"/>
+    <cellStyle name="Percent 2 20" xfId="259" xr:uid="{00000000-0005-0000-0000-00001F010000}"/>
+    <cellStyle name="Percent 2 21" xfId="260" xr:uid="{00000000-0005-0000-0000-000020010000}"/>
+    <cellStyle name="Percent 2 22" xfId="261" xr:uid="{00000000-0005-0000-0000-000021010000}"/>
+    <cellStyle name="Percent 2 23" xfId="262" xr:uid="{00000000-0005-0000-0000-000022010000}"/>
+    <cellStyle name="Percent 2 24" xfId="263" xr:uid="{00000000-0005-0000-0000-000023010000}"/>
+    <cellStyle name="Percent 2 25" xfId="264" xr:uid="{00000000-0005-0000-0000-000024010000}"/>
+    <cellStyle name="Percent 2 3" xfId="47" xr:uid="{00000000-0005-0000-0000-000025010000}"/>
+    <cellStyle name="Percent 2 4" xfId="48" xr:uid="{00000000-0005-0000-0000-000026010000}"/>
+    <cellStyle name="Percent 2 5" xfId="49" xr:uid="{00000000-0005-0000-0000-000027010000}"/>
+    <cellStyle name="Percent 2 6" xfId="265" xr:uid="{00000000-0005-0000-0000-000028010000}"/>
+    <cellStyle name="Percent 2 7" xfId="266" xr:uid="{00000000-0005-0000-0000-000029010000}"/>
+    <cellStyle name="Percent 2 8" xfId="267" xr:uid="{00000000-0005-0000-0000-00002A010000}"/>
+    <cellStyle name="Percent 2 9" xfId="268" xr:uid="{00000000-0005-0000-0000-00002B010000}"/>
+    <cellStyle name="Percent 3" xfId="50" xr:uid="{00000000-0005-0000-0000-00002C010000}"/>
+    <cellStyle name="Percent 3 2" xfId="51" xr:uid="{00000000-0005-0000-0000-00002D010000}"/>
+    <cellStyle name="Percent 3 3" xfId="52" xr:uid="{00000000-0005-0000-0000-00002E010000}"/>
+    <cellStyle name="Percent 3 4" xfId="53" xr:uid="{00000000-0005-0000-0000-00002F010000}"/>
+    <cellStyle name="Percent 3 5" xfId="54" xr:uid="{00000000-0005-0000-0000-000030010000}"/>
+    <cellStyle name="Percent 4" xfId="55" xr:uid="{00000000-0005-0000-0000-000031010000}"/>
+    <cellStyle name="TableStyleLight1" xfId="269" xr:uid="{00000000-0005-0000-0000-000032010000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -6036,7 +6042,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -6069,9 +6075,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -6104,6 +6127,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -6279,7 +6319,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -6661,7 +6701,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr codeName="Sheet38">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -6753,7 +6793,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr codeName="Sheet43">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -6845,7 +6885,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr codeName="Sheet31">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -9624,7 +9664,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet32">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -10431,7 +10471,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr codeName="Sheet44">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -14151,7 +14191,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr codeName="Sheet21">
     <tabColor rgb="FF7030A0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -14769,7 +14809,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr codeName="Sheet45">
     <tabColor rgb="FF7030A0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -16453,7 +16493,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <sheetPr codeName="Sheet6">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -16491,77 +16531,77 @@
       <c r="A2" s="216" t="s">
         <v>646</v>
       </c>
-      <c r="B2" s="305" t="s">
+      <c r="B2" s="307" t="s">
         <v>1078</v>
       </c>
-      <c r="C2" s="306"/>
-      <c r="D2" s="307"/>
-      <c r="E2" s="305" t="s">
+      <c r="C2" s="308"/>
+      <c r="D2" s="309"/>
+      <c r="E2" s="307" t="s">
         <v>1079</v>
       </c>
-      <c r="F2" s="306"/>
-      <c r="G2" s="307"/>
-      <c r="H2" s="305" t="s">
+      <c r="F2" s="308"/>
+      <c r="G2" s="309"/>
+      <c r="H2" s="307" t="s">
         <v>1080</v>
       </c>
-      <c r="I2" s="306"/>
-      <c r="J2" s="307"/>
+      <c r="I2" s="308"/>
+      <c r="J2" s="309"/>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A3" s="302" t="s">
+      <c r="A3" s="303" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="302" t="s">
+      <c r="B3" s="303" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="302" t="s">
+      <c r="C3" s="303" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="302" t="s">
+      <c r="D3" s="303" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="302" t="s">
+      <c r="E3" s="303" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="302" t="s">
+      <c r="F3" s="303" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="302" t="s">
+      <c r="G3" s="303" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="308" t="s">
+      <c r="H3" s="306" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="308" t="s">
+      <c r="I3" s="306" t="s">
         <v>90</v>
       </c>
-      <c r="J3" s="308" t="s">
+      <c r="J3" s="306" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A4" s="303"/>
-      <c r="B4" s="303"/>
-      <c r="C4" s="303"/>
-      <c r="D4" s="303"/>
-      <c r="E4" s="303"/>
-      <c r="F4" s="303"/>
-      <c r="G4" s="303"/>
-      <c r="H4" s="308"/>
-      <c r="I4" s="308"/>
-      <c r="J4" s="308"/>
+      <c r="A4" s="304"/>
+      <c r="B4" s="304"/>
+      <c r="C4" s="304"/>
+      <c r="D4" s="304"/>
+      <c r="E4" s="304"/>
+      <c r="F4" s="304"/>
+      <c r="G4" s="304"/>
+      <c r="H4" s="306"/>
+      <c r="I4" s="306"/>
+      <c r="J4" s="306"/>
     </row>
     <row r="5" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A5" s="304"/>
-      <c r="B5" s="304"/>
-      <c r="C5" s="304"/>
-      <c r="D5" s="304"/>
-      <c r="E5" s="304"/>
-      <c r="F5" s="304"/>
-      <c r="G5" s="304"/>
-      <c r="H5" s="302"/>
-      <c r="I5" s="302"/>
-      <c r="J5" s="302"/>
+      <c r="A5" s="305"/>
+      <c r="B5" s="305"/>
+      <c r="C5" s="305"/>
+      <c r="D5" s="305"/>
+      <c r="E5" s="305"/>
+      <c r="F5" s="305"/>
+      <c r="G5" s="305"/>
+      <c r="H5" s="303"/>
+      <c r="I5" s="303"/>
+      <c r="J5" s="303"/>
     </row>
     <row r="6" spans="1:10" ht="12.75">
       <c r="A6" s="101">
@@ -17554,54 +17594,49 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="11.25" customHeight="1">
-      <c r="A37" s="329" t="s">
+      <c r="A37" s="302" t="s">
         <v>115</v>
       </c>
-      <c r="B37" s="329"/>
-      <c r="C37" s="329"/>
-      <c r="D37" s="329"/>
-      <c r="E37" s="329"/>
-      <c r="F37" s="329"/>
-      <c r="G37" s="329"/>
-      <c r="H37" s="329"/>
-      <c r="I37" s="329"/>
-      <c r="J37" s="329"/>
+      <c r="B37" s="302"/>
+      <c r="C37" s="302"/>
+      <c r="D37" s="302"/>
+      <c r="E37" s="302"/>
+      <c r="F37" s="302"/>
+      <c r="G37" s="302"/>
+      <c r="H37" s="302"/>
+      <c r="I37" s="302"/>
+      <c r="J37" s="302"/>
     </row>
     <row r="38" spans="1:10" ht="24.75" customHeight="1">
-      <c r="A38" s="329" t="s">
+      <c r="A38" s="302" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="329"/>
-      <c r="C38" s="329"/>
-      <c r="D38" s="329"/>
-      <c r="E38" s="329"/>
-      <c r="F38" s="329"/>
-      <c r="G38" s="329"/>
-      <c r="H38" s="329"/>
-      <c r="I38" s="329"/>
-      <c r="J38" s="329"/>
+      <c r="B38" s="302"/>
+      <c r="C38" s="302"/>
+      <c r="D38" s="302"/>
+      <c r="E38" s="302"/>
+      <c r="F38" s="302"/>
+      <c r="G38" s="302"/>
+      <c r="H38" s="302"/>
+      <c r="I38" s="302"/>
+      <c r="J38" s="302"/>
     </row>
     <row r="39" spans="1:10" ht="11.25" customHeight="1">
-      <c r="A39" s="329" t="s">
+      <c r="A39" s="302" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="329"/>
-      <c r="C39" s="329"/>
-      <c r="D39" s="329"/>
-      <c r="E39" s="329"/>
-      <c r="F39" s="329"/>
-      <c r="G39" s="329"/>
-      <c r="H39" s="329"/>
-      <c r="I39" s="329"/>
-      <c r="J39" s="329"/>
+      <c r="B39" s="302"/>
+      <c r="C39" s="302"/>
+      <c r="D39" s="302"/>
+      <c r="E39" s="302"/>
+      <c r="F39" s="302"/>
+      <c r="G39" s="302"/>
+      <c r="H39" s="302"/>
+      <c r="I39" s="302"/>
+      <c r="J39" s="302"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A38:J38"/>
-    <mergeCell ref="A39:J39"/>
-    <mergeCell ref="G3:G5"/>
-    <mergeCell ref="H3:H5"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="F3:F5"/>
     <mergeCell ref="A3:A5"/>
@@ -17614,6 +17649,11 @@
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A37:J37"/>
+    <mergeCell ref="A38:J38"/>
+    <mergeCell ref="A39:J39"/>
+    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="H3:H5"/>
   </mergeCells>
   <pageMargins left="0.9055118110236221" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId1"/>
@@ -17621,7 +17661,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr codeName="Sheet42">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -17653,83 +17693,83 @@
       <c r="G1" s="290"/>
       <c r="H1" s="290"/>
       <c r="I1" s="290"/>
-      <c r="J1" s="309"/>
+      <c r="J1" s="310"/>
     </row>
     <row r="2" spans="1:10" ht="25.5" customHeight="1">
       <c r="A2" s="216" t="s">
         <v>646</v>
       </c>
-      <c r="B2" s="305" t="s">
+      <c r="B2" s="307" t="s">
         <v>1081</v>
       </c>
-      <c r="C2" s="306"/>
-      <c r="D2" s="307"/>
-      <c r="E2" s="308" t="s">
+      <c r="C2" s="308"/>
+      <c r="D2" s="309"/>
+      <c r="E2" s="306" t="s">
         <v>1082</v>
       </c>
-      <c r="F2" s="308"/>
-      <c r="G2" s="308"/>
-      <c r="H2" s="308" t="s">
+      <c r="F2" s="306"/>
+      <c r="G2" s="306"/>
+      <c r="H2" s="306" t="s">
         <v>1083</v>
       </c>
-      <c r="I2" s="308"/>
-      <c r="J2" s="308"/>
+      <c r="I2" s="306"/>
+      <c r="J2" s="306"/>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A3" s="302" t="s">
+      <c r="A3" s="303" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="302" t="s">
+      <c r="B3" s="303" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="302" t="s">
+      <c r="C3" s="303" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="302" t="s">
+      <c r="D3" s="303" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="302" t="s">
+      <c r="E3" s="303" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="302" t="s">
+      <c r="F3" s="303" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="302" t="s">
+      <c r="G3" s="303" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="308" t="s">
+      <c r="H3" s="306" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="308" t="s">
+      <c r="I3" s="306" t="s">
         <v>90</v>
       </c>
-      <c r="J3" s="308" t="s">
+      <c r="J3" s="306" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A4" s="303"/>
-      <c r="B4" s="303"/>
-      <c r="C4" s="303"/>
-      <c r="D4" s="303"/>
-      <c r="E4" s="303"/>
-      <c r="F4" s="303"/>
-      <c r="G4" s="303"/>
-      <c r="H4" s="308"/>
-      <c r="I4" s="308"/>
-      <c r="J4" s="308"/>
+      <c r="A4" s="304"/>
+      <c r="B4" s="304"/>
+      <c r="C4" s="304"/>
+      <c r="D4" s="304"/>
+      <c r="E4" s="304"/>
+      <c r="F4" s="304"/>
+      <c r="G4" s="304"/>
+      <c r="H4" s="306"/>
+      <c r="I4" s="306"/>
+      <c r="J4" s="306"/>
     </row>
     <row r="5" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A5" s="304"/>
-      <c r="B5" s="304"/>
-      <c r="C5" s="304"/>
-      <c r="D5" s="304"/>
-      <c r="E5" s="304"/>
-      <c r="F5" s="304"/>
-      <c r="G5" s="304"/>
-      <c r="H5" s="302"/>
-      <c r="I5" s="302"/>
-      <c r="J5" s="302"/>
+      <c r="A5" s="305"/>
+      <c r="B5" s="305"/>
+      <c r="C5" s="305"/>
+      <c r="D5" s="305"/>
+      <c r="E5" s="305"/>
+      <c r="F5" s="305"/>
+      <c r="G5" s="305"/>
+      <c r="H5" s="303"/>
+      <c r="I5" s="303"/>
+      <c r="J5" s="303"/>
     </row>
     <row r="6" spans="1:10" ht="12.75">
       <c r="A6" s="101">
@@ -18722,54 +18762,49 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="11.25" customHeight="1">
-      <c r="A37" s="329" t="s">
+      <c r="A37" s="302" t="s">
         <v>115</v>
       </c>
-      <c r="B37" s="329"/>
-      <c r="C37" s="329"/>
-      <c r="D37" s="329"/>
-      <c r="E37" s="329"/>
-      <c r="F37" s="329"/>
-      <c r="G37" s="329"/>
-      <c r="H37" s="329"/>
-      <c r="I37" s="329"/>
-      <c r="J37" s="329"/>
+      <c r="B37" s="302"/>
+      <c r="C37" s="302"/>
+      <c r="D37" s="302"/>
+      <c r="E37" s="302"/>
+      <c r="F37" s="302"/>
+      <c r="G37" s="302"/>
+      <c r="H37" s="302"/>
+      <c r="I37" s="302"/>
+      <c r="J37" s="302"/>
     </row>
     <row r="38" spans="1:10" ht="24" customHeight="1">
-      <c r="A38" s="329" t="s">
+      <c r="A38" s="302" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="329"/>
-      <c r="C38" s="329"/>
-      <c r="D38" s="329"/>
-      <c r="E38" s="329"/>
-      <c r="F38" s="329"/>
-      <c r="G38" s="329"/>
-      <c r="H38" s="329"/>
-      <c r="I38" s="329"/>
-      <c r="J38" s="329"/>
+      <c r="B38" s="302"/>
+      <c r="C38" s="302"/>
+      <c r="D38" s="302"/>
+      <c r="E38" s="302"/>
+      <c r="F38" s="302"/>
+      <c r="G38" s="302"/>
+      <c r="H38" s="302"/>
+      <c r="I38" s="302"/>
+      <c r="J38" s="302"/>
     </row>
     <row r="39" spans="1:10" ht="11.25" customHeight="1">
-      <c r="A39" s="329" t="s">
+      <c r="A39" s="302" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="329"/>
-      <c r="C39" s="329"/>
-      <c r="D39" s="329"/>
-      <c r="E39" s="329"/>
-      <c r="F39" s="329"/>
-      <c r="G39" s="329"/>
-      <c r="H39" s="329"/>
-      <c r="I39" s="329"/>
-      <c r="J39" s="329"/>
+      <c r="B39" s="302"/>
+      <c r="C39" s="302"/>
+      <c r="D39" s="302"/>
+      <c r="E39" s="302"/>
+      <c r="F39" s="302"/>
+      <c r="G39" s="302"/>
+      <c r="H39" s="302"/>
+      <c r="I39" s="302"/>
+      <c r="J39" s="302"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="A37:J37"/>
     <mergeCell ref="A38:J38"/>
     <mergeCell ref="A39:J39"/>
     <mergeCell ref="G3:G5"/>
@@ -18782,6 +18817,11 @@
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="E3:E5"/>
     <mergeCell ref="F3:F5"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="A37:J37"/>
   </mergeCells>
   <pageMargins left="0.9055118110236221" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId1"/>
@@ -18789,7 +18829,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <sheetPr codeName="Sheet46">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -18821,83 +18861,83 @@
       <c r="G1" s="290"/>
       <c r="H1" s="290"/>
       <c r="I1" s="290"/>
-      <c r="J1" s="309"/>
+      <c r="J1" s="310"/>
     </row>
     <row r="2" spans="1:10" ht="25.5" customHeight="1">
       <c r="A2" s="216" t="s">
         <v>646</v>
       </c>
-      <c r="B2" s="308" t="s">
+      <c r="B2" s="306" t="s">
         <v>1084</v>
       </c>
-      <c r="C2" s="308"/>
-      <c r="D2" s="308"/>
-      <c r="E2" s="308" t="s">
+      <c r="C2" s="306"/>
+      <c r="D2" s="306"/>
+      <c r="E2" s="306" t="s">
         <v>1085</v>
       </c>
-      <c r="F2" s="308"/>
-      <c r="G2" s="308"/>
-      <c r="H2" s="308" t="s">
+      <c r="F2" s="306"/>
+      <c r="G2" s="306"/>
+      <c r="H2" s="306" t="s">
         <v>1086</v>
       </c>
-      <c r="I2" s="308"/>
-      <c r="J2" s="308"/>
+      <c r="I2" s="306"/>
+      <c r="J2" s="306"/>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A3" s="312" t="s">
+      <c r="A3" s="311" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="308" t="s">
+      <c r="B3" s="306" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="308" t="s">
+      <c r="C3" s="306" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="308" t="s">
+      <c r="D3" s="306" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="308" t="s">
+      <c r="E3" s="306" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="308" t="s">
+      <c r="F3" s="306" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="308" t="s">
+      <c r="G3" s="306" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="308" t="s">
+      <c r="H3" s="306" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="308" t="s">
+      <c r="I3" s="306" t="s">
         <v>90</v>
       </c>
-      <c r="J3" s="308" t="s">
+      <c r="J3" s="306" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A4" s="312"/>
-      <c r="B4" s="308"/>
-      <c r="C4" s="308"/>
-      <c r="D4" s="308"/>
-      <c r="E4" s="308"/>
-      <c r="F4" s="308"/>
-      <c r="G4" s="308"/>
-      <c r="H4" s="308"/>
-      <c r="I4" s="308"/>
-      <c r="J4" s="308"/>
+      <c r="A4" s="311"/>
+      <c r="B4" s="306"/>
+      <c r="C4" s="306"/>
+      <c r="D4" s="306"/>
+      <c r="E4" s="306"/>
+      <c r="F4" s="306"/>
+      <c r="G4" s="306"/>
+      <c r="H4" s="306"/>
+      <c r="I4" s="306"/>
+      <c r="J4" s="306"/>
     </row>
     <row r="5" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A5" s="313"/>
-      <c r="B5" s="302"/>
-      <c r="C5" s="302"/>
-      <c r="D5" s="302"/>
-      <c r="E5" s="302"/>
-      <c r="F5" s="302"/>
-      <c r="G5" s="302"/>
-      <c r="H5" s="302"/>
-      <c r="I5" s="302"/>
-      <c r="J5" s="302"/>
+      <c r="A5" s="312"/>
+      <c r="B5" s="303"/>
+      <c r="C5" s="303"/>
+      <c r="D5" s="303"/>
+      <c r="E5" s="303"/>
+      <c r="F5" s="303"/>
+      <c r="G5" s="303"/>
+      <c r="H5" s="303"/>
+      <c r="I5" s="303"/>
+      <c r="J5" s="303"/>
     </row>
     <row r="6" spans="1:10" ht="12.75">
       <c r="A6" s="101">
@@ -19890,54 +19930,49 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="11.25" customHeight="1">
-      <c r="A37" s="329" t="s">
+      <c r="A37" s="302" t="s">
         <v>1087</v>
       </c>
-      <c r="B37" s="329"/>
-      <c r="C37" s="329"/>
-      <c r="D37" s="329"/>
-      <c r="E37" s="329"/>
-      <c r="F37" s="329"/>
-      <c r="G37" s="329"/>
-      <c r="H37" s="329"/>
-      <c r="I37" s="329"/>
-      <c r="J37" s="329"/>
+      <c r="B37" s="302"/>
+      <c r="C37" s="302"/>
+      <c r="D37" s="302"/>
+      <c r="E37" s="302"/>
+      <c r="F37" s="302"/>
+      <c r="G37" s="302"/>
+      <c r="H37" s="302"/>
+      <c r="I37" s="302"/>
+      <c r="J37" s="302"/>
     </row>
     <row r="38" spans="1:10" ht="21.75" customHeight="1">
-      <c r="A38" s="329" t="s">
+      <c r="A38" s="302" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="329"/>
-      <c r="C38" s="329"/>
-      <c r="D38" s="329"/>
-      <c r="E38" s="329"/>
-      <c r="F38" s="329"/>
-      <c r="G38" s="329"/>
-      <c r="H38" s="329"/>
-      <c r="I38" s="329"/>
-      <c r="J38" s="329"/>
+      <c r="B38" s="302"/>
+      <c r="C38" s="302"/>
+      <c r="D38" s="302"/>
+      <c r="E38" s="302"/>
+      <c r="F38" s="302"/>
+      <c r="G38" s="302"/>
+      <c r="H38" s="302"/>
+      <c r="I38" s="302"/>
+      <c r="J38" s="302"/>
     </row>
     <row r="39" spans="1:10" ht="11.25" customHeight="1">
-      <c r="A39" s="329" t="s">
+      <c r="A39" s="302" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="329"/>
-      <c r="C39" s="329"/>
-      <c r="D39" s="329"/>
-      <c r="E39" s="329"/>
-      <c r="F39" s="329"/>
-      <c r="G39" s="329"/>
-      <c r="H39" s="329"/>
-      <c r="I39" s="329"/>
-      <c r="J39" s="329"/>
+      <c r="B39" s="302"/>
+      <c r="C39" s="302"/>
+      <c r="D39" s="302"/>
+      <c r="E39" s="302"/>
+      <c r="F39" s="302"/>
+      <c r="G39" s="302"/>
+      <c r="H39" s="302"/>
+      <c r="I39" s="302"/>
+      <c r="J39" s="302"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="A37:J37"/>
     <mergeCell ref="A38:J38"/>
     <mergeCell ref="A39:J39"/>
     <mergeCell ref="G3:G5"/>
@@ -19950,6 +19985,11 @@
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="E3:E5"/>
     <mergeCell ref="F3:F5"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="A37:J37"/>
   </mergeCells>
   <pageMargins left="0.9055118110236221" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="85" orientation="portrait" r:id="rId1"/>
@@ -19957,7 +19997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet10">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -20471,7 +20511,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <sheetPr codeName="Sheet52">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -20492,94 +20532,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="29.25" customHeight="1">
-      <c r="A1" s="314" t="s">
+      <c r="A1" s="313" t="s">
         <v>1014</v>
       </c>
-      <c r="B1" s="315"/>
-      <c r="C1" s="315"/>
-      <c r="D1" s="315"/>
-      <c r="E1" s="315"/>
-      <c r="F1" s="315"/>
-      <c r="G1" s="315"/>
-      <c r="H1" s="315"/>
-      <c r="I1" s="315"/>
-      <c r="J1" s="316"/>
+      <c r="B1" s="314"/>
+      <c r="C1" s="314"/>
+      <c r="D1" s="314"/>
+      <c r="E1" s="314"/>
+      <c r="F1" s="314"/>
+      <c r="G1" s="314"/>
+      <c r="H1" s="314"/>
+      <c r="I1" s="314"/>
+      <c r="J1" s="315"/>
     </row>
     <row r="2" spans="1:10" ht="25.5" customHeight="1">
       <c r="A2" s="216" t="s">
         <v>646</v>
       </c>
-      <c r="B2" s="305" t="s">
+      <c r="B2" s="307" t="s">
         <v>1088</v>
       </c>
-      <c r="C2" s="306"/>
-      <c r="D2" s="307"/>
-      <c r="E2" s="305" t="s">
+      <c r="C2" s="308"/>
+      <c r="D2" s="309"/>
+      <c r="E2" s="307" t="s">
         <v>1089</v>
       </c>
-      <c r="F2" s="306"/>
-      <c r="G2" s="307"/>
-      <c r="H2" s="305" t="s">
+      <c r="F2" s="308"/>
+      <c r="G2" s="309"/>
+      <c r="H2" s="307" t="s">
         <v>1090</v>
       </c>
-      <c r="I2" s="306"/>
-      <c r="J2" s="307"/>
+      <c r="I2" s="308"/>
+      <c r="J2" s="309"/>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A3" s="302" t="s">
+      <c r="A3" s="303" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="302" t="s">
+      <c r="B3" s="303" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="302" t="s">
+      <c r="C3" s="303" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="302" t="s">
+      <c r="D3" s="303" t="s">
         <v>1091</v>
       </c>
-      <c r="E3" s="302" t="s">
+      <c r="E3" s="303" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="302" t="s">
+      <c r="F3" s="303" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="302" t="s">
+      <c r="G3" s="303" t="s">
         <v>1092</v>
       </c>
-      <c r="H3" s="302" t="s">
+      <c r="H3" s="303" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="302" t="s">
+      <c r="I3" s="303" t="s">
         <v>90</v>
       </c>
-      <c r="J3" s="302" t="s">
+      <c r="J3" s="303" t="s">
         <v>1092</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A4" s="303"/>
-      <c r="B4" s="303"/>
-      <c r="C4" s="303"/>
-      <c r="D4" s="303"/>
-      <c r="E4" s="303"/>
-      <c r="F4" s="303"/>
-      <c r="G4" s="303"/>
-      <c r="H4" s="303"/>
-      <c r="I4" s="303"/>
-      <c r="J4" s="303"/>
+      <c r="A4" s="304"/>
+      <c r="B4" s="304"/>
+      <c r="C4" s="304"/>
+      <c r="D4" s="304"/>
+      <c r="E4" s="304"/>
+      <c r="F4" s="304"/>
+      <c r="G4" s="304"/>
+      <c r="H4" s="304"/>
+      <c r="I4" s="304"/>
+      <c r="J4" s="304"/>
     </row>
     <row r="5" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A5" s="304"/>
-      <c r="B5" s="304"/>
-      <c r="C5" s="304"/>
-      <c r="D5" s="304"/>
-      <c r="E5" s="304"/>
-      <c r="F5" s="304"/>
-      <c r="G5" s="304"/>
-      <c r="H5" s="304"/>
-      <c r="I5" s="304"/>
-      <c r="J5" s="304"/>
+      <c r="A5" s="305"/>
+      <c r="B5" s="305"/>
+      <c r="C5" s="305"/>
+      <c r="D5" s="305"/>
+      <c r="E5" s="305"/>
+      <c r="F5" s="305"/>
+      <c r="G5" s="305"/>
+      <c r="H5" s="305"/>
+      <c r="I5" s="305"/>
+      <c r="J5" s="305"/>
     </row>
     <row r="6" spans="1:10" ht="12.75">
       <c r="A6" s="101">
@@ -21572,32 +21612,32 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="11.25" customHeight="1">
-      <c r="A37" s="329" t="s">
+      <c r="A37" s="302" t="s">
         <v>115</v>
       </c>
-      <c r="B37" s="329"/>
-      <c r="C37" s="329"/>
-      <c r="D37" s="329"/>
-      <c r="E37" s="329"/>
-      <c r="F37" s="329"/>
-      <c r="G37" s="329"/>
-      <c r="H37" s="329"/>
-      <c r="I37" s="329"/>
-      <c r="J37" s="329"/>
+      <c r="B37" s="302"/>
+      <c r="C37" s="302"/>
+      <c r="D37" s="302"/>
+      <c r="E37" s="302"/>
+      <c r="F37" s="302"/>
+      <c r="G37" s="302"/>
+      <c r="H37" s="302"/>
+      <c r="I37" s="302"/>
+      <c r="J37" s="302"/>
     </row>
     <row r="38" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A38" s="329" t="s">
+      <c r="A38" s="302" t="s">
         <v>18</v>
       </c>
-      <c r="B38" s="329"/>
-      <c r="C38" s="329"/>
-      <c r="D38" s="329"/>
-      <c r="E38" s="329"/>
-      <c r="F38" s="329"/>
-      <c r="G38" s="329"/>
-      <c r="H38" s="329"/>
-      <c r="I38" s="329"/>
-      <c r="J38" s="329"/>
+      <c r="B38" s="302"/>
+      <c r="C38" s="302"/>
+      <c r="D38" s="302"/>
+      <c r="E38" s="302"/>
+      <c r="F38" s="302"/>
+      <c r="G38" s="302"/>
+      <c r="H38" s="302"/>
+      <c r="I38" s="302"/>
+      <c r="J38" s="302"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -21624,7 +21664,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <sheetPr codeName="Sheet47">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -21643,37 +21683,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="323" t="s">
+      <c r="A1" s="322" t="s">
         <v>1038</v>
       </c>
-      <c r="B1" s="323"/>
-      <c r="C1" s="323"/>
-      <c r="D1" s="323"/>
-      <c r="E1" s="323"/>
-      <c r="F1" s="323"/>
-      <c r="G1" s="323"/>
-      <c r="H1" s="323"/>
+      <c r="B1" s="322"/>
+      <c r="C1" s="322"/>
+      <c r="D1" s="322"/>
+      <c r="E1" s="322"/>
+      <c r="F1" s="322"/>
+      <c r="G1" s="322"/>
+      <c r="H1" s="322"/>
     </row>
     <row r="2" spans="1:8" ht="24.75" customHeight="1">
-      <c r="A2" s="324" t="s">
+      <c r="A2" s="323" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="326" t="s">
+      <c r="B2" s="325" t="s">
         <v>1093</v>
       </c>
-      <c r="C2" s="326"/>
-      <c r="D2" s="326"/>
-      <c r="E2" s="342" t="s">
+      <c r="C2" s="325"/>
+      <c r="D2" s="325"/>
+      <c r="E2" s="326" t="s">
         <v>146</v>
       </c>
-      <c r="F2" s="343"/>
-      <c r="G2" s="344"/>
-      <c r="H2" s="324" t="s">
+      <c r="F2" s="327"/>
+      <c r="G2" s="328"/>
+      <c r="H2" s="323" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="325"/>
+      <c r="A3" s="324"/>
       <c r="B3" s="217" t="s">
         <v>20</v>
       </c>
@@ -21692,7 +21732,7 @@
       <c r="G3" s="217" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="325"/>
+      <c r="H3" s="324"/>
     </row>
     <row r="4" spans="1:8" customFormat="1" ht="15">
       <c r="A4" s="109" t="s">
@@ -36203,52 +36243,52 @@
       </c>
     </row>
     <row r="562" spans="1:8">
-      <c r="A562" s="320" t="s">
+      <c r="A562" s="319" t="s">
         <v>14</v>
       </c>
-      <c r="B562" s="321"/>
-      <c r="C562" s="321"/>
-      <c r="D562" s="321"/>
-      <c r="E562" s="321"/>
-      <c r="F562" s="321"/>
-      <c r="G562" s="321"/>
-      <c r="H562" s="322"/>
+      <c r="B562" s="320"/>
+      <c r="C562" s="320"/>
+      <c r="D562" s="320"/>
+      <c r="E562" s="320"/>
+      <c r="F562" s="320"/>
+      <c r="G562" s="320"/>
+      <c r="H562" s="321"/>
     </row>
     <row r="563" spans="1:8" ht="21" customHeight="1">
-      <c r="A563" s="317" t="s">
+      <c r="A563" s="316" t="s">
         <v>22</v>
       </c>
-      <c r="B563" s="318"/>
-      <c r="C563" s="318"/>
-      <c r="D563" s="318"/>
-      <c r="E563" s="318"/>
-      <c r="F563" s="318"/>
-      <c r="G563" s="318"/>
-      <c r="H563" s="319"/>
+      <c r="B563" s="317"/>
+      <c r="C563" s="317"/>
+      <c r="D563" s="317"/>
+      <c r="E563" s="317"/>
+      <c r="F563" s="317"/>
+      <c r="G563" s="317"/>
+      <c r="H563" s="318"/>
     </row>
     <row r="564" spans="1:8" ht="12" customHeight="1">
-      <c r="A564" s="317" t="s">
+      <c r="A564" s="316" t="s">
         <v>23</v>
       </c>
-      <c r="B564" s="318"/>
-      <c r="C564" s="318"/>
-      <c r="D564" s="318"/>
-      <c r="E564" s="318"/>
-      <c r="F564" s="318"/>
-      <c r="G564" s="318"/>
-      <c r="H564" s="319"/>
+      <c r="B564" s="317"/>
+      <c r="C564" s="317"/>
+      <c r="D564" s="317"/>
+      <c r="E564" s="317"/>
+      <c r="F564" s="317"/>
+      <c r="G564" s="317"/>
+      <c r="H564" s="318"/>
     </row>
     <row r="565" spans="1:8" ht="12" customHeight="1">
-      <c r="A565" s="317" t="s">
+      <c r="A565" s="316" t="s">
         <v>359</v>
       </c>
-      <c r="B565" s="318"/>
-      <c r="C565" s="318"/>
-      <c r="D565" s="318"/>
-      <c r="E565" s="318"/>
-      <c r="F565" s="318"/>
-      <c r="G565" s="318"/>
-      <c r="H565" s="319"/>
+      <c r="B565" s="317"/>
+      <c r="C565" s="317"/>
+      <c r="D565" s="317"/>
+      <c r="E565" s="317"/>
+      <c r="F565" s="317"/>
+      <c r="G565" s="317"/>
+      <c r="H565" s="318"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -36269,7 +36309,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <sheetPr codeName="Sheet48">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -36289,24 +36329,24 @@
       <c r="B1" s="290"/>
       <c r="C1" s="290"/>
       <c r="D1" s="290"/>
-      <c r="E1" s="309"/>
+      <c r="E1" s="310"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1">
-      <c r="A2" s="313" t="s">
+      <c r="A2" s="312" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="313" t="s">
+      <c r="B2" s="312" t="s">
         <v>107</v>
       </c>
-      <c r="C2" s="305" t="s">
+      <c r="C2" s="307" t="s">
         <v>150</v>
       </c>
-      <c r="D2" s="306"/>
-      <c r="E2" s="307"/>
+      <c r="D2" s="308"/>
+      <c r="E2" s="309"/>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="328"/>
-      <c r="B3" s="328"/>
+      <c r="A3" s="332"/>
+      <c r="B3" s="332"/>
       <c r="C3" s="215" t="s">
         <v>34</v>
       </c>
@@ -36845,22 +36885,22 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A35" s="329" t="s">
+      <c r="A35" s="302" t="s">
         <v>148</v>
       </c>
-      <c r="B35" s="329"/>
-      <c r="C35" s="329"/>
-      <c r="D35" s="329"/>
-      <c r="E35" s="329"/>
+      <c r="B35" s="302"/>
+      <c r="C35" s="302"/>
+      <c r="D35" s="302"/>
+      <c r="E35" s="302"/>
     </row>
     <row r="36" spans="1:5" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A36" s="310" t="s">
+      <c r="A36" s="329" t="s">
         <v>18</v>
       </c>
-      <c r="B36" s="311"/>
-      <c r="C36" s="311"/>
-      <c r="D36" s="311"/>
-      <c r="E36" s="327"/>
+      <c r="B36" s="330"/>
+      <c r="C36" s="330"/>
+      <c r="D36" s="330"/>
+      <c r="E36" s="331"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -36877,7 +36917,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <sheetPr codeName="Sheet18">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -36891,11 +36931,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1">
-      <c r="A1" s="330" t="s">
+      <c r="A1" s="333" t="s">
         <v>1044</v>
       </c>
-      <c r="B1" s="330"/>
-      <c r="C1" s="330"/>
+      <c r="B1" s="333"/>
+      <c r="C1" s="333"/>
     </row>
     <row r="2" spans="1:3" ht="38.25">
       <c r="A2" s="44" t="s">
@@ -40396,11 +40436,11 @@
       </c>
     </row>
     <row r="320" spans="1:3">
-      <c r="A320" s="345" t="s">
+      <c r="A320" s="334" t="s">
         <v>14</v>
       </c>
-      <c r="B320" s="345"/>
-      <c r="C320" s="345"/>
+      <c r="B320" s="334"/>
+      <c r="C320" s="334"/>
     </row>
   </sheetData>
   <sortState ref="B243:C317">
@@ -40419,7 +40459,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <sheetPr codeName="Sheet19">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -40433,11 +40473,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="31.5" customHeight="1">
-      <c r="A1" s="330" t="s">
+      <c r="A1" s="333" t="s">
         <v>1045</v>
       </c>
-      <c r="B1" s="330"/>
-      <c r="C1" s="330"/>
+      <c r="B1" s="333"/>
+      <c r="C1" s="333"/>
     </row>
     <row r="2" spans="1:3" ht="38.25">
       <c r="A2" s="44" t="s">
@@ -43949,11 +43989,11 @@
       </c>
     </row>
     <row r="321" spans="1:3">
-      <c r="A321" s="345" t="s">
+      <c r="A321" s="334" t="s">
         <v>14</v>
       </c>
-      <c r="B321" s="345"/>
-      <c r="C321" s="345"/>
+      <c r="B321" s="334"/>
+      <c r="C321" s="334"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -43966,7 +44006,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <sheetPr codeName="Sheet22">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -43992,24 +44032,24 @@
       <c r="F1" s="271"/>
     </row>
     <row r="2" spans="1:6" ht="21.6" customHeight="1">
-      <c r="A2" s="331" t="s">
+      <c r="A2" s="337" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="332" t="s">
+      <c r="B2" s="338" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="332" t="s">
+      <c r="C2" s="338" t="s">
         <v>145</v>
       </c>
-      <c r="D2" s="335"/>
-      <c r="E2" s="336"/>
-      <c r="F2" s="333" t="s">
+      <c r="D2" s="341"/>
+      <c r="E2" s="342"/>
+      <c r="F2" s="339" t="s">
         <v>1094</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="22.5" customHeight="1">
-      <c r="A3" s="331"/>
-      <c r="B3" s="331"/>
+      <c r="A3" s="337"/>
+      <c r="B3" s="337"/>
       <c r="C3" s="218" t="s">
         <v>4</v>
       </c>
@@ -44019,7 +44059,7 @@
       <c r="E3" s="218" t="s">
         <v>113</v>
       </c>
-      <c r="F3" s="334" t="s">
+      <c r="F3" s="340" t="s">
         <v>87</v>
       </c>
     </row>
@@ -44094,7 +44134,7 @@
         <v>627042</v>
       </c>
       <c r="D7" s="118">
-        <v>1485291</v>
+        <v>485291</v>
       </c>
       <c r="E7" s="118">
         <v>161073</v>
@@ -44124,24 +44164,24 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A9" s="346" t="s">
+      <c r="A9" s="335" t="s">
         <v>144</v>
       </c>
-      <c r="B9" s="346"/>
-      <c r="C9" s="346"/>
-      <c r="D9" s="346"/>
-      <c r="E9" s="346"/>
-      <c r="F9" s="346"/>
+      <c r="B9" s="335"/>
+      <c r="C9" s="335"/>
+      <c r="D9" s="335"/>
+      <c r="E9" s="335"/>
+      <c r="F9" s="335"/>
     </row>
     <row r="10" spans="1:6" ht="15">
-      <c r="A10" s="347" t="s">
+      <c r="A10" s="336" t="s">
         <v>65</v>
       </c>
-      <c r="B10" s="347"/>
-      <c r="C10" s="347"/>
-      <c r="D10" s="347"/>
-      <c r="E10" s="347"/>
-      <c r="F10" s="347"/>
+      <c r="B10" s="336"/>
+      <c r="C10" s="336"/>
+      <c r="D10" s="336"/>
+      <c r="E10" s="336"/>
+      <c r="F10" s="336"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -44159,7 +44199,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <sheetPr codeName="Sheet41">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -44183,25 +44223,25 @@
       <c r="G1" s="270"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1">
-      <c r="A2" s="331" t="s">
+      <c r="A2" s="337" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="331" t="s">
+      <c r="B2" s="337" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="337" t="s">
+      <c r="C2" s="345" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="338"/>
-      <c r="E2" s="339"/>
+      <c r="D2" s="346"/>
+      <c r="E2" s="347"/>
       <c r="F2" s="285" t="s">
         <v>108</v>
       </c>
       <c r="G2" s="287"/>
     </row>
     <row r="3" spans="1:7" ht="31.5" customHeight="1">
-      <c r="A3" s="331"/>
-      <c r="B3" s="331"/>
+      <c r="A3" s="337"/>
+      <c r="B3" s="337"/>
       <c r="C3" s="129" t="s">
         <v>20</v>
       </c>
@@ -44286,37 +44326,37 @@
       </c>
     </row>
     <row r="7" spans="1:7" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A7" s="340" t="s">
+      <c r="A7" s="343" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="341"/>
-      <c r="C7" s="341"/>
-      <c r="D7" s="341"/>
-      <c r="E7" s="341"/>
-      <c r="F7" s="341"/>
-      <c r="G7" s="341"/>
+      <c r="B7" s="344"/>
+      <c r="C7" s="344"/>
+      <c r="D7" s="344"/>
+      <c r="E7" s="344"/>
+      <c r="F7" s="344"/>
+      <c r="G7" s="344"/>
     </row>
     <row r="8" spans="1:7" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A8" s="340" t="s">
+      <c r="A8" s="343" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="341"/>
-      <c r="C8" s="341"/>
-      <c r="D8" s="341"/>
-      <c r="E8" s="341"/>
-      <c r="F8" s="341"/>
-      <c r="G8" s="341"/>
+      <c r="B8" s="344"/>
+      <c r="C8" s="344"/>
+      <c r="D8" s="344"/>
+      <c r="E8" s="344"/>
+      <c r="F8" s="344"/>
+      <c r="G8" s="344"/>
     </row>
     <row r="9" spans="1:7" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A9" s="340" t="s">
+      <c r="A9" s="343" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="341"/>
-      <c r="C9" s="341"/>
-      <c r="D9" s="341"/>
-      <c r="E9" s="341"/>
-      <c r="F9" s="341"/>
-      <c r="G9" s="341"/>
+      <c r="B9" s="344"/>
+      <c r="C9" s="344"/>
+      <c r="D9" s="344"/>
+      <c r="E9" s="344"/>
+      <c r="F9" s="344"/>
+      <c r="G9" s="344"/>
     </row>
     <row r="12" spans="1:7" ht="35.25" customHeight="1">
       <c r="A12" s="268" t="s">
@@ -44330,25 +44370,25 @@
       <c r="G12" s="270"/>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1">
-      <c r="A13" s="331" t="s">
+      <c r="A13" s="337" t="s">
         <v>111</v>
       </c>
-      <c r="B13" s="331" t="s">
+      <c r="B13" s="337" t="s">
         <v>109</v>
       </c>
-      <c r="C13" s="337" t="s">
+      <c r="C13" s="345" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="338"/>
-      <c r="E13" s="339"/>
+      <c r="D13" s="346"/>
+      <c r="E13" s="347"/>
       <c r="F13" s="285" t="s">
         <v>108</v>
       </c>
       <c r="G13" s="287"/>
     </row>
     <row r="14" spans="1:7" ht="31.5" customHeight="1">
-      <c r="A14" s="331"/>
-      <c r="B14" s="331"/>
+      <c r="A14" s="337"/>
+      <c r="B14" s="337"/>
       <c r="C14" s="129" t="s">
         <v>20</v>
       </c>
@@ -44433,40 +44473,45 @@
       </c>
     </row>
     <row r="18" spans="1:7" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A18" s="340" t="s">
+      <c r="A18" s="343" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="341"/>
-      <c r="C18" s="341"/>
-      <c r="D18" s="341"/>
-      <c r="E18" s="341"/>
-      <c r="F18" s="341"/>
-      <c r="G18" s="341"/>
+      <c r="B18" s="344"/>
+      <c r="C18" s="344"/>
+      <c r="D18" s="344"/>
+      <c r="E18" s="344"/>
+      <c r="F18" s="344"/>
+      <c r="G18" s="344"/>
     </row>
     <row r="19" spans="1:7" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A19" s="340" t="s">
+      <c r="A19" s="343" t="s">
         <v>166</v>
       </c>
-      <c r="B19" s="341"/>
-      <c r="C19" s="341"/>
-      <c r="D19" s="341"/>
-      <c r="E19" s="341"/>
-      <c r="F19" s="341"/>
-      <c r="G19" s="341"/>
+      <c r="B19" s="344"/>
+      <c r="C19" s="344"/>
+      <c r="D19" s="344"/>
+      <c r="E19" s="344"/>
+      <c r="F19" s="344"/>
+      <c r="G19" s="344"/>
     </row>
     <row r="20" spans="1:7" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A20" s="340" t="s">
+      <c r="A20" s="343" t="s">
         <v>168</v>
       </c>
-      <c r="B20" s="341"/>
-      <c r="C20" s="341"/>
-      <c r="D20" s="341"/>
-      <c r="E20" s="341"/>
-      <c r="F20" s="341"/>
-      <c r="G20" s="341"/>
+      <c r="B20" s="344"/>
+      <c r="C20" s="344"/>
+      <c r="D20" s="344"/>
+      <c r="E20" s="344"/>
+      <c r="F20" s="344"/>
+      <c r="G20" s="344"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:E2"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A9:G9"/>
@@ -44478,11 +44523,6 @@
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="F13:G13"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="97" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -44490,7 +44530,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet11">
     <tabColor rgb="FF7030A0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -44507,12 +44547,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="244" t="s">
+      <c r="A1" s="239" t="s">
         <v>1050</v>
       </c>
-      <c r="B1" s="245"/>
-      <c r="C1" s="245"/>
-      <c r="D1" s="246"/>
+      <c r="B1" s="244"/>
+      <c r="C1" s="244"/>
+      <c r="D1" s="245"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="154" t="s">
@@ -44521,10 +44561,10 @@
       <c r="B2" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="249" t="s">
+      <c r="C2" s="248" t="s">
         <v>151</v>
       </c>
-      <c r="D2" s="250"/>
+      <c r="D2" s="249"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="67">
@@ -44533,10 +44573,10 @@
       <c r="B3" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="239">
+      <c r="C3" s="250">
         <v>1.18</v>
       </c>
-      <c r="D3" s="240"/>
+      <c r="D3" s="251"/>
       <c r="E3" s="36"/>
     </row>
     <row r="4" spans="1:5">
@@ -44546,10 +44586,10 @@
       <c r="B4" s="68" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="239">
+      <c r="C4" s="250">
         <v>9.9</v>
       </c>
-      <c r="D4" s="240"/>
+      <c r="D4" s="251"/>
       <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1">
@@ -44559,19 +44599,19 @@
       <c r="B5" s="68" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="239">
+      <c r="C5" s="250">
         <v>5.89</v>
       </c>
-      <c r="D5" s="240"/>
+      <c r="D5" s="251"/>
       <c r="E5" s="36"/>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="251" t="s">
+      <c r="A6" s="252" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="251"/>
-      <c r="C6" s="251"/>
-      <c r="D6" s="251"/>
+      <c r="B6" s="252"/>
+      <c r="C6" s="252"/>
+      <c r="D6" s="252"/>
       <c r="E6" s="37"/>
     </row>
     <row r="7" spans="1:5">
@@ -44582,12 +44622,12 @@
       <c r="E7" s="37"/>
     </row>
     <row r="8" spans="1:5" s="37" customFormat="1" ht="27" customHeight="1">
-      <c r="A8" s="244" t="s">
+      <c r="A8" s="239" t="s">
         <v>1051</v>
       </c>
-      <c r="B8" s="245"/>
-      <c r="C8" s="245"/>
-      <c r="D8" s="246"/>
+      <c r="B8" s="244"/>
+      <c r="C8" s="244"/>
+      <c r="D8" s="245"/>
       <c r="E8" s="35"/>
     </row>
     <row r="9" spans="1:5" s="37" customFormat="1">
@@ -44597,10 +44637,10 @@
       <c r="B9" s="155" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="249" t="s">
+      <c r="C9" s="248" t="s">
         <v>151</v>
       </c>
-      <c r="D9" s="250"/>
+      <c r="D9" s="249"/>
       <c r="E9" s="35"/>
     </row>
     <row r="10" spans="1:5" s="37" customFormat="1" ht="15" customHeight="1">
@@ -44610,10 +44650,10 @@
       <c r="B10" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="239">
+      <c r="C10" s="250">
         <v>5.61</v>
       </c>
-      <c r="D10" s="240"/>
+      <c r="D10" s="251"/>
       <c r="E10" s="38"/>
     </row>
     <row r="11" spans="1:5" s="37" customFormat="1" ht="15" customHeight="1">
@@ -44623,10 +44663,10 @@
       <c r="B11" s="68" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="239">
+      <c r="C11" s="250">
         <v>9.41</v>
       </c>
-      <c r="D11" s="240"/>
+      <c r="D11" s="251"/>
       <c r="E11" s="38"/>
     </row>
     <row r="12" spans="1:5" s="37" customFormat="1" ht="15" customHeight="1">
@@ -44636,19 +44676,19 @@
       <c r="B12" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="239">
+      <c r="C12" s="250">
         <v>6.05</v>
       </c>
-      <c r="D12" s="240"/>
+      <c r="D12" s="251"/>
       <c r="E12" s="36"/>
     </row>
     <row r="13" spans="1:5" s="37" customFormat="1">
-      <c r="A13" s="241" t="s">
+      <c r="A13" s="253" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="242"/>
-      <c r="C13" s="242"/>
-      <c r="D13" s="243"/>
+      <c r="B13" s="254"/>
+      <c r="C13" s="254"/>
+      <c r="D13" s="255"/>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="29"/>
@@ -44658,13 +44698,13 @@
       <c r="E14" s="37"/>
     </row>
     <row r="15" spans="1:5" ht="27.75" customHeight="1">
-      <c r="A15" s="252" t="s">
+      <c r="A15" s="256" t="s">
         <v>1067</v>
       </c>
-      <c r="B15" s="253"/>
-      <c r="C15" s="253"/>
-      <c r="D15" s="253"/>
-      <c r="E15" s="253"/>
+      <c r="B15" s="257"/>
+      <c r="C15" s="257"/>
+      <c r="D15" s="257"/>
+      <c r="E15" s="257"/>
     </row>
     <row r="16" spans="1:5" ht="25.5">
       <c r="A16" s="156" t="s">
@@ -44735,13 +44775,13 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="18.75" customHeight="1">
-      <c r="A20" s="247" t="s">
+      <c r="A20" s="242" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="247"/>
-      <c r="C20" s="247"/>
-      <c r="D20" s="247"/>
-      <c r="E20" s="256"/>
+      <c r="B20" s="242"/>
+      <c r="C20" s="242"/>
+      <c r="D20" s="242"/>
+      <c r="E20" s="247"/>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="39"/>
@@ -44750,13 +44790,13 @@
       <c r="D21" s="30"/>
     </row>
     <row r="22" spans="1:5" ht="27" customHeight="1">
-      <c r="A22" s="244" t="s">
+      <c r="A22" s="239" t="s">
         <v>1068</v>
       </c>
-      <c r="B22" s="254"/>
-      <c r="C22" s="254"/>
-      <c r="D22" s="254"/>
-      <c r="E22" s="255"/>
+      <c r="B22" s="240"/>
+      <c r="C22" s="240"/>
+      <c r="D22" s="240"/>
+      <c r="E22" s="241"/>
     </row>
     <row r="23" spans="1:5" ht="25.5">
       <c r="A23" s="156" t="s">
@@ -44827,13 +44867,13 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A27" s="247" t="s">
+      <c r="A27" s="242" t="s">
         <v>114</v>
       </c>
-      <c r="B27" s="247"/>
-      <c r="C27" s="247"/>
-      <c r="D27" s="247"/>
-      <c r="E27" s="247"/>
+      <c r="B27" s="242"/>
+      <c r="C27" s="242"/>
+      <c r="D27" s="242"/>
+      <c r="E27" s="242"/>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="39"/>
@@ -44842,13 +44882,13 @@
       <c r="D28" s="30"/>
     </row>
     <row r="29" spans="1:5" ht="32.25" customHeight="1">
-      <c r="A29" s="257" t="s">
+      <c r="A29" s="246" t="s">
         <v>1069</v>
       </c>
-      <c r="B29" s="257"/>
-      <c r="C29" s="257"/>
-      <c r="D29" s="257"/>
-      <c r="E29" s="257"/>
+      <c r="B29" s="246"/>
+      <c r="C29" s="246"/>
+      <c r="D29" s="246"/>
+      <c r="E29" s="246"/>
     </row>
     <row r="30" spans="1:5" ht="25.5">
       <c r="A30" s="156" t="s">
@@ -44919,13 +44959,13 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A34" s="247" t="s">
+      <c r="A34" s="242" t="s">
         <v>114</v>
       </c>
-      <c r="B34" s="247"/>
-      <c r="C34" s="247"/>
-      <c r="D34" s="247"/>
-      <c r="E34" s="247"/>
+      <c r="B34" s="242"/>
+      <c r="C34" s="242"/>
+      <c r="D34" s="242"/>
+      <c r="E34" s="242"/>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="39"/>
@@ -44934,13 +44974,13 @@
       <c r="D35" s="30"/>
     </row>
     <row r="36" spans="1:5" ht="27" customHeight="1">
-      <c r="A36" s="257" t="s">
+      <c r="A36" s="246" t="s">
         <v>1070</v>
       </c>
-      <c r="B36" s="257"/>
-      <c r="C36" s="257"/>
-      <c r="D36" s="257"/>
-      <c r="E36" s="257"/>
+      <c r="B36" s="246"/>
+      <c r="C36" s="246"/>
+      <c r="D36" s="246"/>
+      <c r="E36" s="246"/>
     </row>
     <row r="37" spans="1:5" ht="25.5">
       <c r="A37" s="156" t="s">
@@ -45011,13 +45051,13 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="12.75" customHeight="1">
-      <c r="A41" s="247" t="s">
+      <c r="A41" s="242" t="s">
         <v>114</v>
       </c>
-      <c r="B41" s="247"/>
-      <c r="C41" s="247"/>
-      <c r="D41" s="247"/>
-      <c r="E41" s="256"/>
+      <c r="B41" s="242"/>
+      <c r="C41" s="242"/>
+      <c r="D41" s="242"/>
+      <c r="E41" s="247"/>
     </row>
     <row r="42" spans="1:5" ht="12.75" customHeight="1">
       <c r="A42" s="170"/>
@@ -45026,12 +45066,12 @@
       <c r="D42" s="170"/>
     </row>
     <row r="43" spans="1:5" ht="30.75" customHeight="1">
-      <c r="A43" s="244" t="s">
+      <c r="A43" s="239" t="s">
         <v>991</v>
       </c>
-      <c r="B43" s="245"/>
-      <c r="C43" s="245"/>
-      <c r="D43" s="246"/>
+      <c r="B43" s="244"/>
+      <c r="C43" s="244"/>
+      <c r="D43" s="245"/>
     </row>
     <row r="44" spans="1:5" ht="30.75" customHeight="1">
       <c r="A44" s="157" t="s">
@@ -45088,12 +45128,12 @@
       </c>
     </row>
     <row r="48" spans="1:5" s="37" customFormat="1">
-      <c r="A48" s="247" t="s">
+      <c r="A48" s="242" t="s">
         <v>42</v>
       </c>
-      <c r="B48" s="248"/>
-      <c r="C48" s="248"/>
-      <c r="D48" s="248"/>
+      <c r="B48" s="243"/>
+      <c r="C48" s="243"/>
+      <c r="D48" s="243"/>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="39"/>
@@ -45102,12 +45142,12 @@
       <c r="D49" s="30"/>
     </row>
     <row r="50" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A50" s="244" t="s">
+      <c r="A50" s="239" t="s">
         <v>992</v>
       </c>
-      <c r="B50" s="245"/>
-      <c r="C50" s="245"/>
-      <c r="D50" s="246"/>
+      <c r="B50" s="244"/>
+      <c r="C50" s="244"/>
+      <c r="D50" s="245"/>
     </row>
     <row r="51" spans="1:4" ht="30.75">
       <c r="A51" s="157" t="s">
@@ -45192,12 +45232,12 @@
       </c>
     </row>
     <row r="57" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A57" s="247" t="s">
+      <c r="A57" s="242" t="s">
         <v>42</v>
       </c>
-      <c r="B57" s="248"/>
-      <c r="C57" s="248"/>
-      <c r="D57" s="248"/>
+      <c r="B57" s="243"/>
+      <c r="C57" s="243"/>
+      <c r="D57" s="243"/>
     </row>
     <row r="58" spans="1:4" ht="12.75" customHeight="1">
       <c r="A58" s="29"/>
@@ -45206,12 +45246,12 @@
       <c r="D58" s="29"/>
     </row>
     <row r="59" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A59" s="244" t="s">
+      <c r="A59" s="239" t="s">
         <v>993</v>
       </c>
-      <c r="B59" s="245"/>
-      <c r="C59" s="245"/>
-      <c r="D59" s="246"/>
+      <c r="B59" s="244"/>
+      <c r="C59" s="244"/>
+      <c r="D59" s="245"/>
     </row>
     <row r="60" spans="1:4" ht="30.75" customHeight="1">
       <c r="A60" s="157" t="s">
@@ -45268,12 +45308,12 @@
       </c>
     </row>
     <row r="64" spans="1:4" s="37" customFormat="1">
-      <c r="A64" s="247" t="s">
+      <c r="A64" s="242" t="s">
         <v>43</v>
       </c>
-      <c r="B64" s="248"/>
-      <c r="C64" s="248"/>
-      <c r="D64" s="248"/>
+      <c r="B64" s="243"/>
+      <c r="C64" s="243"/>
+      <c r="D64" s="243"/>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="29"/>
@@ -45282,12 +45322,12 @@
       <c r="D65" s="29"/>
     </row>
     <row r="66" spans="1:4" ht="27.75" customHeight="1">
-      <c r="A66" s="244" t="s">
+      <c r="A66" s="239" t="s">
         <v>994</v>
       </c>
-      <c r="B66" s="245"/>
-      <c r="C66" s="245"/>
-      <c r="D66" s="246"/>
+      <c r="B66" s="244"/>
+      <c r="C66" s="244"/>
+      <c r="D66" s="245"/>
     </row>
     <row r="67" spans="1:4" ht="30.75">
       <c r="A67" s="157" t="s">
@@ -45372,12 +45412,12 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="12.75" customHeight="1">
-      <c r="A73" s="247" t="s">
+      <c r="A73" s="242" t="s">
         <v>43</v>
       </c>
-      <c r="B73" s="248"/>
-      <c r="C73" s="248"/>
-      <c r="D73" s="248"/>
+      <c r="B73" s="243"/>
+      <c r="C73" s="243"/>
+      <c r="D73" s="243"/>
     </row>
     <row r="74" spans="1:4" ht="12.75" customHeight="1">
       <c r="A74" s="170"/>
@@ -45386,12 +45426,12 @@
       <c r="D74" s="33"/>
     </row>
     <row r="75" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A75" s="244" t="s">
+      <c r="A75" s="239" t="s">
         <v>995</v>
       </c>
-      <c r="B75" s="245"/>
-      <c r="C75" s="245"/>
-      <c r="D75" s="246"/>
+      <c r="B75" s="244"/>
+      <c r="C75" s="244"/>
+      <c r="D75" s="245"/>
     </row>
     <row r="76" spans="1:4" ht="30.75" customHeight="1">
       <c r="A76" s="157" t="s">
@@ -45448,12 +45488,12 @@
       </c>
     </row>
     <row r="80" spans="1:4" s="37" customFormat="1">
-      <c r="A80" s="247" t="s">
+      <c r="A80" s="242" t="s">
         <v>116</v>
       </c>
-      <c r="B80" s="248"/>
-      <c r="C80" s="248"/>
-      <c r="D80" s="248"/>
+      <c r="B80" s="243"/>
+      <c r="C80" s="243"/>
+      <c r="D80" s="243"/>
     </row>
     <row r="81" spans="1:4" ht="12.75" customHeight="1">
       <c r="A81" s="170"/>
@@ -45462,12 +45502,12 @@
       <c r="D81" s="33"/>
     </row>
     <row r="82" spans="1:4" ht="32.25" customHeight="1">
-      <c r="A82" s="244" t="s">
+      <c r="A82" s="239" t="s">
         <v>996</v>
       </c>
-      <c r="B82" s="245"/>
-      <c r="C82" s="245"/>
-      <c r="D82" s="246"/>
+      <c r="B82" s="244"/>
+      <c r="C82" s="244"/>
+      <c r="D82" s="245"/>
     </row>
     <row r="83" spans="1:4" ht="30.75">
       <c r="A83" s="157" t="s">
@@ -45552,12 +45592,12 @@
       </c>
     </row>
     <row r="89" spans="1:4">
-      <c r="A89" s="247" t="s">
+      <c r="A89" s="242" t="s">
         <v>116</v>
       </c>
-      <c r="B89" s="248"/>
-      <c r="C89" s="248"/>
-      <c r="D89" s="248"/>
+      <c r="B89" s="243"/>
+      <c r="C89" s="243"/>
+      <c r="D89" s="243"/>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="40"/>
@@ -45566,12 +45606,12 @@
       <c r="D90" s="34"/>
     </row>
     <row r="91" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A91" s="244" t="s">
+      <c r="A91" s="239" t="s">
         <v>997</v>
       </c>
-      <c r="B91" s="245"/>
-      <c r="C91" s="245"/>
-      <c r="D91" s="246"/>
+      <c r="B91" s="244"/>
+      <c r="C91" s="244"/>
+      <c r="D91" s="245"/>
     </row>
     <row r="92" spans="1:4" ht="30.75" customHeight="1">
       <c r="A92" s="157" t="s">
@@ -45628,12 +45668,12 @@
       </c>
     </row>
     <row r="96" spans="1:4" s="37" customFormat="1">
-      <c r="A96" s="247" t="s">
+      <c r="A96" s="242" t="s">
         <v>42</v>
       </c>
-      <c r="B96" s="248"/>
-      <c r="C96" s="248"/>
-      <c r="D96" s="248"/>
+      <c r="B96" s="243"/>
+      <c r="C96" s="243"/>
+      <c r="D96" s="243"/>
     </row>
     <row r="97" spans="1:5">
       <c r="A97" s="40"/>
@@ -45648,12 +45688,12 @@
       <c r="D98" s="34"/>
     </row>
     <row r="99" spans="1:5" ht="31.5" customHeight="1">
-      <c r="A99" s="244" t="s">
+      <c r="A99" s="239" t="s">
         <v>998</v>
       </c>
-      <c r="B99" s="245"/>
-      <c r="C99" s="245"/>
-      <c r="D99" s="246"/>
+      <c r="B99" s="244"/>
+      <c r="C99" s="244"/>
+      <c r="D99" s="245"/>
     </row>
     <row r="100" spans="1:5" ht="30.75">
       <c r="A100" s="157" t="s">
@@ -45739,12 +45779,12 @@
       </c>
     </row>
     <row r="106" spans="1:5">
-      <c r="A106" s="247" t="s">
+      <c r="A106" s="242" t="s">
         <v>42</v>
       </c>
-      <c r="B106" s="248"/>
-      <c r="C106" s="248"/>
-      <c r="D106" s="248"/>
+      <c r="B106" s="243"/>
+      <c r="C106" s="243"/>
+      <c r="D106" s="243"/>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" s="189"/>
@@ -45753,12 +45793,12 @@
       <c r="D107" s="190"/>
     </row>
     <row r="108" spans="1:5" ht="30.75" customHeight="1">
-      <c r="A108" s="244" t="s">
+      <c r="A108" s="239" t="s">
         <v>999</v>
       </c>
-      <c r="B108" s="245"/>
-      <c r="C108" s="245"/>
-      <c r="D108" s="246"/>
+      <c r="B108" s="244"/>
+      <c r="C108" s="244"/>
+      <c r="D108" s="245"/>
     </row>
     <row r="109" spans="1:5" ht="30.75" customHeight="1">
       <c r="A109" s="157" t="s">
@@ -45815,20 +45855,20 @@
       </c>
     </row>
     <row r="113" spans="1:4" s="37" customFormat="1">
-      <c r="A113" s="247" t="s">
+      <c r="A113" s="242" t="s">
         <v>43</v>
       </c>
-      <c r="B113" s="248"/>
-      <c r="C113" s="248"/>
-      <c r="D113" s="248"/>
+      <c r="B113" s="243"/>
+      <c r="C113" s="243"/>
+      <c r="D113" s="243"/>
     </row>
     <row r="115" spans="1:4" ht="31.5" customHeight="1">
-      <c r="A115" s="244" t="s">
+      <c r="A115" s="239" t="s">
         <v>1000</v>
       </c>
-      <c r="B115" s="245"/>
-      <c r="C115" s="245"/>
-      <c r="D115" s="246"/>
+      <c r="B115" s="244"/>
+      <c r="C115" s="244"/>
+      <c r="D115" s="245"/>
     </row>
     <row r="116" spans="1:4" ht="30.75">
       <c r="A116" s="157" t="s">
@@ -45913,12 +45953,12 @@
       </c>
     </row>
     <row r="122" spans="1:4">
-      <c r="A122" s="247" t="s">
+      <c r="A122" s="242" t="s">
         <v>43</v>
       </c>
-      <c r="B122" s="248"/>
-      <c r="C122" s="248"/>
-      <c r="D122" s="248"/>
+      <c r="B122" s="243"/>
+      <c r="C122" s="243"/>
+      <c r="D122" s="243"/>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="189"/>
@@ -45927,12 +45967,12 @@
       <c r="D123" s="190"/>
     </row>
     <row r="124" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A124" s="244" t="s">
+      <c r="A124" s="239" t="s">
         <v>1001</v>
       </c>
-      <c r="B124" s="245"/>
-      <c r="C124" s="245"/>
-      <c r="D124" s="246"/>
+      <c r="B124" s="244"/>
+      <c r="C124" s="244"/>
+      <c r="D124" s="245"/>
     </row>
     <row r="125" spans="1:4" ht="30.75" customHeight="1">
       <c r="A125" s="157" t="s">
@@ -45989,20 +46029,20 @@
       </c>
     </row>
     <row r="129" spans="1:4" s="37" customFormat="1">
-      <c r="A129" s="247" t="s">
+      <c r="A129" s="242" t="s">
         <v>116</v>
       </c>
-      <c r="B129" s="248"/>
-      <c r="C129" s="248"/>
-      <c r="D129" s="248"/>
+      <c r="B129" s="243"/>
+      <c r="C129" s="243"/>
+      <c r="D129" s="243"/>
     </row>
     <row r="131" spans="1:4" ht="31.5" customHeight="1">
-      <c r="A131" s="244" t="s">
+      <c r="A131" s="239" t="s">
         <v>1002</v>
       </c>
-      <c r="B131" s="245"/>
-      <c r="C131" s="245"/>
-      <c r="D131" s="246"/>
+      <c r="B131" s="244"/>
+      <c r="C131" s="244"/>
+      <c r="D131" s="245"/>
     </row>
     <row r="132" spans="1:4" ht="30.75">
       <c r="A132" s="157" t="s">
@@ -46087,12 +46127,12 @@
       </c>
     </row>
     <row r="138" spans="1:4">
-      <c r="A138" s="247" t="s">
+      <c r="A138" s="242" t="s">
         <v>116</v>
       </c>
-      <c r="B138" s="248"/>
-      <c r="C138" s="248"/>
-      <c r="D138" s="248"/>
+      <c r="B138" s="243"/>
+      <c r="C138" s="243"/>
+      <c r="D138" s="243"/>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="189"/>
@@ -46101,12 +46141,12 @@
       <c r="D139" s="190"/>
     </row>
     <row r="140" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A140" s="244" t="s">
+      <c r="A140" s="239" t="s">
         <v>1003</v>
       </c>
-      <c r="B140" s="245"/>
-      <c r="C140" s="245"/>
-      <c r="D140" s="246"/>
+      <c r="B140" s="244"/>
+      <c r="C140" s="244"/>
+      <c r="D140" s="245"/>
     </row>
     <row r="141" spans="1:4" ht="30.75" customHeight="1">
       <c r="A141" s="157" t="s">
@@ -46163,12 +46203,12 @@
       </c>
     </row>
     <row r="145" spans="1:4" s="37" customFormat="1">
-      <c r="A145" s="247" t="s">
+      <c r="A145" s="242" t="s">
         <v>42</v>
       </c>
-      <c r="B145" s="248"/>
-      <c r="C145" s="248"/>
-      <c r="D145" s="248"/>
+      <c r="B145" s="243"/>
+      <c r="C145" s="243"/>
+      <c r="D145" s="243"/>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="189"/>
@@ -46177,12 +46217,12 @@
       <c r="D146" s="190"/>
     </row>
     <row r="148" spans="1:4" ht="30" customHeight="1">
-      <c r="A148" s="244" t="s">
+      <c r="A148" s="239" t="s">
         <v>1004</v>
       </c>
-      <c r="B148" s="245"/>
-      <c r="C148" s="245"/>
-      <c r="D148" s="246"/>
+      <c r="B148" s="244"/>
+      <c r="C148" s="244"/>
+      <c r="D148" s="245"/>
     </row>
     <row r="149" spans="1:4" ht="30.75">
       <c r="A149" s="157" t="s">
@@ -46267,12 +46307,12 @@
       </c>
     </row>
     <row r="155" spans="1:4">
-      <c r="A155" s="247" t="s">
+      <c r="A155" s="242" t="s">
         <v>42</v>
       </c>
-      <c r="B155" s="248"/>
-      <c r="C155" s="248"/>
-      <c r="D155" s="248"/>
+      <c r="B155" s="243"/>
+      <c r="C155" s="243"/>
+      <c r="D155" s="243"/>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="189"/>
@@ -46281,12 +46321,12 @@
       <c r="D156" s="190"/>
     </row>
     <row r="157" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A157" s="244" t="s">
+      <c r="A157" s="239" t="s">
         <v>1005</v>
       </c>
-      <c r="B157" s="245"/>
-      <c r="C157" s="245"/>
-      <c r="D157" s="246"/>
+      <c r="B157" s="244"/>
+      <c r="C157" s="244"/>
+      <c r="D157" s="245"/>
     </row>
     <row r="158" spans="1:4" ht="30.75" customHeight="1">
       <c r="A158" s="157" t="s">
@@ -46343,20 +46383,20 @@
       </c>
     </row>
     <row r="162" spans="1:4" s="37" customFormat="1">
-      <c r="A162" s="247" t="s">
+      <c r="A162" s="242" t="s">
         <v>43</v>
       </c>
-      <c r="B162" s="248"/>
-      <c r="C162" s="248"/>
-      <c r="D162" s="248"/>
+      <c r="B162" s="243"/>
+      <c r="C162" s="243"/>
+      <c r="D162" s="243"/>
     </row>
     <row r="165" spans="1:4" ht="30" customHeight="1">
-      <c r="A165" s="244" t="s">
+      <c r="A165" s="239" t="s">
         <v>1006</v>
       </c>
-      <c r="B165" s="245"/>
-      <c r="C165" s="245"/>
-      <c r="D165" s="246"/>
+      <c r="B165" s="244"/>
+      <c r="C165" s="244"/>
+      <c r="D165" s="245"/>
     </row>
     <row r="166" spans="1:4" ht="30.75">
       <c r="A166" s="157" t="s">
@@ -46441,12 +46481,12 @@
       </c>
     </row>
     <row r="172" spans="1:4">
-      <c r="A172" s="247" t="s">
+      <c r="A172" s="242" t="s">
         <v>43</v>
       </c>
-      <c r="B172" s="248"/>
-      <c r="C172" s="248"/>
-      <c r="D172" s="248"/>
+      <c r="B172" s="243"/>
+      <c r="C172" s="243"/>
+      <c r="D172" s="243"/>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" s="189"/>
@@ -46455,12 +46495,12 @@
       <c r="D173" s="190"/>
     </row>
     <row r="174" spans="1:4" ht="30.75" customHeight="1">
-      <c r="A174" s="244" t="s">
+      <c r="A174" s="239" t="s">
         <v>1007</v>
       </c>
-      <c r="B174" s="245"/>
-      <c r="C174" s="245"/>
-      <c r="D174" s="246"/>
+      <c r="B174" s="244"/>
+      <c r="C174" s="244"/>
+      <c r="D174" s="245"/>
     </row>
     <row r="175" spans="1:4" ht="30.75" customHeight="1">
       <c r="A175" s="157" t="s">
@@ -46517,20 +46557,20 @@
       </c>
     </row>
     <row r="179" spans="1:4" s="37" customFormat="1">
-      <c r="A179" s="247" t="s">
+      <c r="A179" s="242" t="s">
         <v>116</v>
       </c>
-      <c r="B179" s="248"/>
-      <c r="C179" s="248"/>
-      <c r="D179" s="248"/>
+      <c r="B179" s="243"/>
+      <c r="C179" s="243"/>
+      <c r="D179" s="243"/>
     </row>
     <row r="181" spans="1:4" ht="30" customHeight="1">
-      <c r="A181" s="244" t="s">
+      <c r="A181" s="239" t="s">
         <v>1008</v>
       </c>
-      <c r="B181" s="254"/>
-      <c r="C181" s="254"/>
-      <c r="D181" s="255"/>
+      <c r="B181" s="240"/>
+      <c r="C181" s="240"/>
+      <c r="D181" s="241"/>
     </row>
     <row r="182" spans="1:4" ht="30.75">
       <c r="A182" s="157" t="s">
@@ -46615,29 +46655,41 @@
       </c>
     </row>
     <row r="188" spans="1:4">
-      <c r="A188" s="247" t="s">
+      <c r="A188" s="242" t="s">
         <v>116</v>
       </c>
-      <c r="B188" s="248"/>
-      <c r="C188" s="248"/>
-      <c r="D188" s="248"/>
+      <c r="B188" s="243"/>
+      <c r="C188" s="243"/>
+      <c r="D188" s="243"/>
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="A181:D181"/>
-    <mergeCell ref="A113:D113"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A96:D96"/>
-    <mergeCell ref="A108:D108"/>
-    <mergeCell ref="A124:D124"/>
-    <mergeCell ref="A129:D129"/>
-    <mergeCell ref="A140:D140"/>
-    <mergeCell ref="A179:D179"/>
-    <mergeCell ref="A145:D145"/>
-    <mergeCell ref="A157:D157"/>
-    <mergeCell ref="A162:D162"/>
-    <mergeCell ref="A174:D174"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A131:D131"/>
+    <mergeCell ref="A138:D138"/>
+    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="A122:D122"/>
+    <mergeCell ref="A99:D99"/>
+    <mergeCell ref="A106:D106"/>
+    <mergeCell ref="A73:D73"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A36:E36"/>
@@ -46654,32 +46706,20 @@
     <mergeCell ref="A59:D59"/>
     <mergeCell ref="A64:D64"/>
     <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A131:D131"/>
-    <mergeCell ref="A138:D138"/>
-    <mergeCell ref="A115:D115"/>
-    <mergeCell ref="A122:D122"/>
-    <mergeCell ref="A99:D99"/>
-    <mergeCell ref="A106:D106"/>
-    <mergeCell ref="A73:D73"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A181:D181"/>
+    <mergeCell ref="A113:D113"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="A108:D108"/>
+    <mergeCell ref="A124:D124"/>
+    <mergeCell ref="A129:D129"/>
+    <mergeCell ref="A140:D140"/>
+    <mergeCell ref="A179:D179"/>
+    <mergeCell ref="A145:D145"/>
+    <mergeCell ref="A157:D157"/>
+    <mergeCell ref="A162:D162"/>
+    <mergeCell ref="A174:D174"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup scale="21" orientation="portrait" r:id="rId1"/>
@@ -46688,7 +46728,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet14">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -48969,7 +49009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet15">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -49545,7 +49585,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet16">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -51763,7 +51803,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet17">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -52251,7 +52291,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet39">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -53311,7 +53351,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr codeName="Sheet40">
     <tabColor rgb="FF7030A0"/>
   </sheetPr>

</xml_diff>